<commit_message>
chore(tracking): the plan's first Changelog row names its PR (#632)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="173">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -546,6 +546,9 @@
   </si>
   <si>
     <t>The first plan: conversations.conversation_archived and conversations.conversation_unarchived, with a conversations.conversation snapshot (the reference flow of ADR 0020).</t>
+  </si>
+  <si>
+    <t>#632</t>
   </si>
 </sst>
 </file>
@@ -2085,6 +2088,9 @@
       <c r="C2" s="3" t="s">
         <v>171</v>
       </c>
+      <c r="D2" s="3" t="s">
+        <v>172</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D2"/>

</xml_diff>

<commit_message>
chore(tracking): name PR #650 in the plan's changelog (#325)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2101" uniqueCount="786">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2102" uniqueCount="787">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -2388,6 +2388,9 @@
   </si>
   <si>
     <t>The conversations module instrumented (campbooks-cloud#325): 40 events for flags, streams, labels, needs, drafts and sends, taught rules and their runs, suggestions, person notes, provider batches, the model pass, Scout's reads and inboxes; records draft, need, rule and rule_run; Coverage for every operation, job, schedule and handler of the module.</t>
+  </si>
+  <si>
+    <t>#650</t>
   </si>
 </sst>
 </file>
@@ -10608,6 +10611,9 @@
       <c r="C3" s="3" t="s">
         <v>785</v>
       </c>
+      <c r="D3" s="3" t="s">
+        <v>786</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D3"/>

</xml_diff>

<commit_message>
chore(tracking): name PR #654 in plan version 3's changelog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3349" uniqueCount="1142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3350" uniqueCount="1143">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -3456,6 +3456,9 @@
   </si>
   <si>
     <t>The identity module instrumented (campbooks-cloud#326): 27 events for sign-ins succeeded and refused, accounts created, sessions ended, ways in and passkeys added and removed, suspensions, workspace and registered apps, consents, held mailbox grants, and token exchanges, reuse and revocation; records account, session, way_in, passkey, client and consent; Coverage for every operation, handler and schedule of the module.</t>
+  </si>
+  <si>
+    <t>#654</t>
   </si>
 </sst>
 </file>
@@ -16171,6 +16174,9 @@
       <c r="C4" s="3" t="s">
         <v>1141</v>
       </c>
+      <c r="D4" s="3" t="s">
+        <v>1142</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D4"/>

</xml_diff>

<commit_message>
chore(tracking): name PR #655 in plan version 4's changelog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3524" uniqueCount="1207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3525" uniqueCount="1208">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -3651,6 +3651,9 @@
   </si>
   <si>
     <t>The web BFF instrumented (campbooks-cloud#327): 3 events for web sessions started, ended one at a time (logging out, signing in again, a copied cookie, outdated scopes, a refused refresh, unreadable tokens, an expired access token) and ended at once (back-channel logout, signing out everywhere, a suspension); the enums of how they end; Coverage for every operation, handler and schedule of the BFF. bff is a platform module, generated into the kernel and tracked from the server.</t>
+  </si>
+  <si>
+    <t>#655</t>
   </si>
 </sst>
 </file>
@@ -17016,6 +17019,9 @@
       <c r="C5" s="3" t="s">
         <v>1206</v>
       </c>
+      <c r="D5" s="3" t="s">
+        <v>1207</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D5"/>

</xml_diff>

<commit_message>
chore(tracking): name PR #657 in plan version 5's changelog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4233" uniqueCount="1409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4234" uniqueCount="1410">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -4257,6 +4257,9 @@
   </si>
   <si>
     <t>The workspaces module instrumented (campbooks-cloud#328): 16 events for workspaces created, updated, deleted and purged, members joined, role changed, left, suspended and unsuspended, invitations created, signup requests filed, approved and rejected, and signup codes minted, revoked and redeemed; records workspace, member, invitation, signup_request and signup_code; Coverage for every operation, handler and job of the module; the conversations and identity exemptions name workspaces.workspace_deleted.</t>
+  </si>
+  <si>
+    <t>#657</t>
   </si>
 </sst>
 </file>
@@ -20151,6 +20154,9 @@
       <c r="C6" s="3" t="s">
         <v>1408</v>
       </c>
+      <c r="D6" s="3" t="s">
+        <v>1409</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D6"/>

</xml_diff>

<commit_message>
fix(workspaces): track a suspension only when it changes the member's state
Postgres keeps microseconds, so a replay's time never equalled the change
recorded: compare whether the member is suspended instead.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -1238,7 +1238,7 @@
     <t>A member's account was suspended: whatever acts in their name in the workspace stops until it is lifted. Tracked in each workspace they belong to.</t>
   </si>
   <si>
-    <t>workspaces.announce_member_suspended announces identity.account_suspended in the workspace, in the transaction that publishes workspaces.member_suspended there; a replay of the change announced already, or an older change, tracks nothing.</t>
+    <t>workspaces.announce_member_suspended announces identity.account_suspended in the workspace, in the transaction that publishes workspaces.member_suspended there; a change that leaves them as they were (a replay, an older change, a second suspension with no lift between) tracks nothing.</t>
   </si>
   <si>
     <t>workspaces.member_unsuspended</t>
@@ -1247,7 +1247,7 @@
     <t>A member's suspension was lifted. Tracked in each workspace they belong to.</t>
   </si>
   <si>
-    <t>workspaces.announce_member_unsuspended announces identity.account_unsuspended in the workspace, likewise; a replay or an older change tracks nothing.</t>
+    <t>workspaces.announce_member_unsuspended announces identity.account_unsuspended in the workspace, likewise; a lift that leaves them as they were (a replay, an older change) tracks nothing.</t>
   </si>
   <si>
     <t>workspaces.signup_code_minted</t>

</xml_diff>

<commit_message>
chore(tracking): name PR #659 in the connectors patch
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5010" uniqueCount="1659">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5011" uniqueCount="1660">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -5007,6 +5007,9 @@
   </si>
   <si>
     <t>The connectors module instrumented (campbooks-cloud#329): 10 events for connections added, reconnected, removed, their health changed and a sync asked for, sync runs (one summary per run, with counts), the outbound changes a run made (counts by end), calendar changes completed, and sends succeeded or failed; records connection, stream and send; Coverage for every operation, job, schedule and handler of the module; the identity operations that hand it a grant name the connection events.</t>
+  </si>
+  <si>
+    <t>#659</t>
   </si>
 </sst>
 </file>
@@ -23689,6 +23692,9 @@
       <c r="C7" s="3" t="s">
         <v>1658</v>
       </c>
+      <c r="D7" s="3" t="s">
+        <v>1659</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D7"/>

</xml_diff>

<commit_message>
chore(tracking): the plan's changelog names PR #661
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6018" uniqueCount="2013">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6019" uniqueCount="2014">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -6069,6 +6069,9 @@
   </si>
   <si>
     <t>The assistant, attention, search and system modules instrumented (campbooks-cloud#330): 15 events for chats with Scout started, continued, answered and deleted, its proposals confirmed, declined and undone, a member's profile updated, an item snoozed and unsnoozed, a workspace's daily AI limit reached, and (the kernel's queue, from the system admin actions) a dead job retried or discarded, a kind's dead jobs retried and a schedule's stuck run discarded; records chat, answer, proposal, profile, item and job; Coverage for every operation, job, schedule and handler of the four modules (search and the telemetry reports exempt).</t>
+  </si>
+  <si>
+    <t>#661</t>
   </si>
 </sst>
 </file>
@@ -28354,6 +28357,9 @@
       <c r="C8" s="3" t="s">
         <v>2012</v>
       </c>
+      <c r="D8" s="3" t="s">
+        <v>2013</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D8"/>

</xml_diff>

<commit_message>
chore(tracking): name PR #662 in the plan changelog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6155" uniqueCount="2057">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6156" uniqueCount="2058">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -6201,6 +6201,9 @@
   </si>
   <si>
     <t>The admin module instrumented (campbooks-cloud#331): 2 instance-wide events for an administrator's profile granted (created or given more permissions) and revoked (permissions taken away or the profile removed) by the server's admin command, as system; record profile and enum permission; no Coverage rows (the module serves no operation and runs no job, schedule or handler).</t>
+  </si>
+  <si>
+    <t>#662</t>
   </si>
 </sst>
 </file>
@@ -28976,6 +28979,9 @@
       <c r="C9" s="3" t="s">
         <v>2056</v>
       </c>
+      <c r="D9" s="3" t="s">
+        <v>2057</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D9"/>

</xml_diff>

<commit_message>
chore(tracking): name the schedule patch's PR (#349)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7082" uniqueCount="2333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7083" uniqueCount="2334">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -7029,6 +7029,9 @@
   </si>
   <si>
     <t>The schedule module instrumented (campbooks-cloud#349): 16 events for events of a calendar created, edited (which fields), moved (the times before), cancelled by a later email, deleted, restored, answered (the answer before), pushed to a provider calendar and unpushed, calendars added by a grant, enabled, disabled, recoloured and removed with their connection, settings updated (which settings), and one summary per batch of a provider's changes applied (counts); records calendar_event, calendar_event_times, calendar and settings; Coverage for every operation, job and handler of the module, apply_outcome and release_delete naming connectors.calendar_change_completed.</t>
+  </si>
+  <si>
+    <t>#663</t>
   </si>
 </sst>
 </file>
@@ -33089,6 +33092,9 @@
       <c r="C10" s="3" t="s">
         <v>2332</v>
       </c>
+      <c r="D10" s="3" t="s">
+        <v>2333</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D10"/>

</xml_diff>

<commit_message>
chore(tracking): the tasks patch names its PR (#665)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6608" uniqueCount="2187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6609" uniqueCount="2188">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -6591,6 +6591,9 @@
   </si>
   <si>
     <t>The tasks module instrumented (campbooks-cloud#340): 8 events for a task created (by a member, or by Scout from an ask), edited (which fields), its due date changed (the date before), planned (the plan before), done, not needed, reopened (the state before) and reassigned (handed off or taken back, with the member who had it); records task, task_due and task_plan; Coverage for every operation, job and handler of the module.</t>
+  </si>
+  <si>
+    <t>#665</t>
   </si>
 </sst>
 </file>
@@ -30972,6 +30975,9 @@
       <c r="C10" s="3" t="s">
         <v>2186</v>
       </c>
+      <c r="D10" s="3" t="s">
+        <v>2187</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D10"/>

</xml_diff>

<commit_message>
chore(tracking): the plan's v11 changelog names #666
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7209" uniqueCount="2389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7210" uniqueCount="2390">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -7197,6 +7197,9 @@
   </si>
   <si>
     <t>Coverage required with no baseline (campbooks-cloud#332): 2 connectors events for an IMAP mailbox's address check asked for again and its message sent or not (with why); Coverage rows for connectors.check_address, connectors.send_address_check and the kernel's maintenance schedules and change-feed sequencer.</t>
+  </si>
+  <si>
+    <t>#666</t>
   </si>
 </sst>
 </file>
@@ -33727,6 +33730,9 @@
       <c r="C11" s="3" t="s">
         <v>2388</v>
       </c>
+      <c r="D11" s="3" t="s">
+        <v>2389</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:D11"/>

</xml_diff>

<commit_message>
fix(tracking): Coverage row for search.on_page_changed, which Pages (#672) added
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Actors!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$245</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Enums!$A$1:$C$426</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Events!$A$1:$L$152</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Properties!$A$1:$K$321</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8087" uniqueCount="2639">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8090" uniqueCount="2641">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -7022,6 +7022,12 @@
     <t>projection of conversations.message_sent: the conversation's entries in the index refreshed</t>
   </si>
   <si>
+    <t>search.on_page_changed</t>
+  </si>
+  <si>
+    <t>projection of pages.page_changed: the page's entry in the index refreshed (removed when trashed or gone)</t>
+  </si>
+  <si>
     <t>search.schedule_workspace_purge</t>
   </si>
   <si>
@@ -7943,7 +7949,7 @@
     <t>#672</t>
   </si>
   <si>
-    <t>Coverage required with no baseline (campbooks-cloud#332): 2 connectors events for an IMAP mailbox's address check asked for again and its message sent or not (with why); Coverage rows for connectors.check_address, connectors.send_address_check and the kernel's maintenance schedules and change-feed sequencer.</t>
+    <t>Coverage required with no baseline (campbooks-cloud#332): 2 connectors events for an IMAP mailbox's address check asked for again and its message sent or not (with why); Coverage rows for connectors.check_address, connectors.send_address_check, search.on_page_changed and the kernel's maintenance schedules and change-feed sequencer.</t>
   </si>
   <si>
     <t>#666</t>
@@ -34721,7 +34727,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D244"/>
+  <dimension ref="A1:D245"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -35224,7 +35230,7 @@
       <c r="B45" s="3" t="s">
         <v>2332</v>
       </c>
-      <c r="C45" s="3" t="s">
+      <c r="D45" s="3" t="s">
         <v>2333</v>
       </c>
     </row>
@@ -35236,7 +35242,7 @@
         <v>2334</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>620</v>
+        <v>2335</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -35244,10 +35250,10 @@
         <v>2261</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>2335</v>
+        <v>2336</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>2336</v>
+        <v>620</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -35258,7 +35264,7 @@
         <v>2337</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>615</v>
+        <v>2338</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -35266,10 +35272,10 @@
         <v>2261</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>2338</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>2265</v>
+        <v>2339</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>615</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -35277,10 +35283,10 @@
         <v>2261</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>2339</v>
-      </c>
-      <c r="C50" s="3" t="s">
-        <v>658</v>
+        <v>2340</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>2265</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -35288,21 +35294,21 @@
         <v>2261</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>2340</v>
+        <v>2341</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>661</v>
+        <v>658</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="3" t="s">
-        <v>484</v>
+        <v>2261</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>2341</v>
-      </c>
-      <c r="D52" s="3" t="s">
         <v>2342</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -35345,8 +35351,8 @@
       <c r="B56" s="3" t="s">
         <v>2349</v>
       </c>
-      <c r="C56" s="3" t="s">
-        <v>144</v>
+      <c r="D56" s="3" t="s">
+        <v>2350</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -35354,10 +35360,10 @@
         <v>484</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>2350</v>
+        <v>2351</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>2351</v>
+        <v>144</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -35379,7 +35385,7 @@
         <v>2354</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>295</v>
+        <v>2355</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -35387,10 +35393,10 @@
         <v>484</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>2355</v>
+        <v>2356</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>359</v>
+        <v>295</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -35398,10 +35404,10 @@
         <v>484</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>2356</v>
-      </c>
-      <c r="D61" s="3" t="s">
         <v>2357</v>
+      </c>
+      <c r="C61" s="3" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -35411,8 +35417,8 @@
       <c r="B62" s="3" t="s">
         <v>2358</v>
       </c>
-      <c r="C62" s="3" t="s">
-        <v>271</v>
+      <c r="D62" s="3" t="s">
+        <v>2359</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -35420,10 +35426,10 @@
         <v>484</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>2359</v>
+        <v>2360</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>300</v>
+        <v>271</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -35431,10 +35437,10 @@
         <v>484</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>2360</v>
-      </c>
-      <c r="D64" s="3" t="s">
         <v>2361</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="65" spans="1:4">
@@ -35466,8 +35472,8 @@
       <c r="B67" s="3" t="s">
         <v>2366</v>
       </c>
-      <c r="C67" s="3" t="s">
-        <v>305</v>
+      <c r="D67" s="3" t="s">
+        <v>2367</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -35475,7 +35481,7 @@
         <v>484</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>2367</v>
+        <v>2368</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>305</v>
@@ -35486,10 +35492,10 @@
         <v>484</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>2368</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>2357</v>
+        <v>2369</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -35497,10 +35503,10 @@
         <v>484</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>2369</v>
-      </c>
-      <c r="C70" s="3" t="s">
         <v>2370</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>2359</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -35510,7 +35516,7 @@
       <c r="B71" s="3" t="s">
         <v>2371</v>
       </c>
-      <c r="D71" s="3" t="s">
+      <c r="C71" s="3" t="s">
         <v>2372</v>
       </c>
     </row>
@@ -35533,7 +35539,7 @@
         <v>2375</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>2357</v>
+        <v>2376</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -35541,10 +35547,10 @@
         <v>484</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>2376</v>
+        <v>2377</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>2377</v>
+        <v>2359</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -35598,8 +35604,8 @@
       <c r="B79" s="3" t="s">
         <v>2386</v>
       </c>
-      <c r="C79" s="3" t="s">
-        <v>149</v>
+      <c r="D79" s="3" t="s">
+        <v>2387</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -35607,10 +35613,10 @@
         <v>484</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>2387</v>
-      </c>
-      <c r="D80" s="3" t="s">
         <v>2388</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -35653,126 +35659,126 @@
       <c r="B84" s="3" t="s">
         <v>2395</v>
       </c>
-      <c r="C84" s="3" t="s">
-        <v>695</v>
+      <c r="D84" s="3" t="s">
+        <v>2396</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="3" t="s">
-        <v>2396</v>
+        <v>484</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>2397</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>2398</v>
+        <v>695</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>2399</v>
       </c>
-      <c r="D86" s="3" t="s">
+      <c r="C86" s="3" t="s">
         <v>2400</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>2401</v>
       </c>
-      <c r="C87" s="3" t="s">
-        <v>85</v>
+      <c r="D87" s="3" t="s">
+        <v>2402</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>2403</v>
+        <v>85</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>2404</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>89</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>2405</v>
+        <v>2406</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>2398</v>
+        <v>89</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>2406</v>
+        <v>2407</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>93</v>
+        <v>2400</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>2407</v>
+        <v>2408</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>2408</v>
+        <v>2409</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>2409</v>
+        <v>2410</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>2410</v>
+        <v>2411</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>121</v>
@@ -35780,10 +35786,10 @@
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>2411</v>
+        <v>2412</v>
       </c>
       <c r="C96" s="3" t="s">
         <v>121</v>
@@ -35791,10 +35797,10 @@
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>2412</v>
+        <v>2413</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>121</v>
@@ -35802,10 +35808,10 @@
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>2413</v>
+        <v>2414</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>121</v>
@@ -35813,10 +35819,10 @@
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>2414</v>
+        <v>2415</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>121</v>
@@ -35824,10 +35830,10 @@
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>2415</v>
+        <v>2416</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>121</v>
@@ -35835,10 +35841,10 @@
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>2416</v>
+        <v>2417</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>121</v>
@@ -35846,10 +35852,10 @@
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>2417</v>
+        <v>2418</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>121</v>
@@ -35857,10 +35863,10 @@
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>2418</v>
+        <v>2419</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>121</v>
@@ -35868,54 +35874,54 @@
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>2419</v>
+        <v>2420</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>2420</v>
+        <v>2421</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>2421</v>
+        <v>132</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>2422</v>
       </c>
-      <c r="D106" s="3" t="s">
+      <c r="C106" s="3" t="s">
         <v>2423</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>2424</v>
       </c>
-      <c r="C107" s="3" t="s">
-        <v>121</v>
+      <c r="D107" s="3" t="s">
+        <v>2425</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>2425</v>
+        <v>2426</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>121</v>
@@ -35923,513 +35929,513 @@
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>2426</v>
+        <v>2427</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>2427</v>
+        <v>2428</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>2428</v>
+        <v>137</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>2429</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>168</v>
+        <v>2430</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>2430</v>
-      </c>
-      <c r="D112" s="3" t="s">
         <v>2431</v>
       </c>
-    </row>
-    <row r="113" spans="1:3">
+      <c r="C112" s="3" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4">
       <c r="A113" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>2432</v>
       </c>
-      <c r="C113" s="3" t="s">
+      <c r="D113" s="3" t="s">
+        <v>2433</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4">
+      <c r="A114" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B114" s="3" t="s">
+        <v>2434</v>
+      </c>
+      <c r="C114" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="114" spans="1:3">
-      <c r="A114" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B114" s="3" t="s">
-        <v>2433</v>
-      </c>
-      <c r="C114" s="3" t="s">
+    <row r="115" spans="1:4">
+      <c r="A115" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B115" s="3" t="s">
+        <v>2435</v>
+      </c>
+      <c r="C115" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="115" spans="1:3">
-      <c r="A115" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B115" s="3" t="s">
-        <v>2434</v>
-      </c>
-      <c r="C115" s="3" t="s">
+    <row r="116" spans="1:4">
+      <c r="A116" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B116" s="3" t="s">
+        <v>2436</v>
+      </c>
+      <c r="C116" s="3" t="s">
         <v>348</v>
       </c>
     </row>
-    <row r="116" spans="1:3">
-      <c r="A116" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B116" s="3" t="s">
-        <v>2435</v>
-      </c>
-      <c r="C116" s="3" t="s">
+    <row r="117" spans="1:4">
+      <c r="A117" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B117" s="3" t="s">
+        <v>2437</v>
+      </c>
+      <c r="C117" s="3" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="117" spans="1:3">
-      <c r="A117" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>2436</v>
-      </c>
-      <c r="C117" s="3" t="s">
+    <row r="118" spans="1:4">
+      <c r="A118" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B118" s="3" t="s">
+        <v>2438</v>
+      </c>
+      <c r="C118" s="3" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="118" spans="1:3">
-      <c r="A118" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B118" s="3" t="s">
-        <v>2437</v>
-      </c>
-      <c r="C118" s="3" t="s">
+    <row r="119" spans="1:4">
+      <c r="A119" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>2439</v>
+      </c>
+      <c r="C119" s="3" t="s">
         <v>343</v>
       </c>
     </row>
-    <row r="119" spans="1:3">
-      <c r="A119" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>2438</v>
-      </c>
-      <c r="C119" s="3" t="s">
+    <row r="120" spans="1:4">
+      <c r="A120" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>2440</v>
+      </c>
+      <c r="C120" s="3" t="s">
         <v>312</v>
       </c>
     </row>
-    <row r="120" spans="1:3">
-      <c r="A120" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>2439</v>
-      </c>
-      <c r="C120" s="3" t="s">
-        <v>2440</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3">
+    <row r="121" spans="1:4">
       <c r="A121" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>2441</v>
       </c>
       <c r="C121" s="3" t="s">
+        <v>2442</v>
+      </c>
+    </row>
+    <row r="122" spans="1:4">
+      <c r="A122" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>2443</v>
+      </c>
+      <c r="C122" s="3" t="s">
         <v>253</v>
       </c>
     </row>
-    <row r="122" spans="1:3">
-      <c r="A122" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B122" s="3" t="s">
-        <v>2442</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>2443</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3">
+    <row r="123" spans="1:4">
       <c r="A123" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>2444</v>
       </c>
       <c r="C123" s="3" t="s">
+        <v>2445</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>2446</v>
+      </c>
+      <c r="C124" s="3" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="124" spans="1:3">
-      <c r="A124" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B124" s="3" t="s">
-        <v>2445</v>
-      </c>
-      <c r="C124" s="3" t="s">
+    <row r="125" spans="1:4">
+      <c r="A125" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>2447</v>
+      </c>
+      <c r="C125" s="3" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="125" spans="1:3">
-      <c r="A125" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B125" s="3" t="s">
-        <v>2446</v>
-      </c>
-      <c r="C125" s="3" t="s">
+    <row r="126" spans="1:4">
+      <c r="A126" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>2448</v>
+      </c>
+      <c r="C126" s="3" t="s">
         <v>324</v>
       </c>
     </row>
-    <row r="126" spans="1:3">
-      <c r="A126" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B126" s="3" t="s">
-        <v>2447</v>
-      </c>
-      <c r="C126" s="3" t="s">
+    <row r="127" spans="1:4">
+      <c r="A127" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>2449</v>
+      </c>
+      <c r="C127" s="3" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="127" spans="1:3">
-      <c r="A127" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B127" s="3" t="s">
-        <v>2448</v>
-      </c>
-      <c r="C127" s="3" t="s">
+    <row r="128" spans="1:4">
+      <c r="A128" s="3" t="s">
+        <v>2398</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>2450</v>
+      </c>
+      <c r="C128" s="3" t="s">
         <v>213</v>
-      </c>
-    </row>
-    <row r="128" spans="1:3">
-      <c r="A128" s="3" t="s">
-        <v>2396</v>
-      </c>
-      <c r="B128" s="3" t="s">
-        <v>2449</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>2450</v>
+        <v>2451</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>2451</v>
+        <v>2452</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>241</v>
+        <v>209</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>2452</v>
-      </c>
-      <c r="D131" s="3" t="s">
         <v>2453</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>2454</v>
       </c>
-      <c r="C132" s="3" t="s">
-        <v>233</v>
+      <c r="D132" s="3" t="s">
+        <v>2455</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>2455</v>
+        <v>2456</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>352</v>
+        <v>233</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>2456</v>
+        <v>2457</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>316</v>
+        <v>352</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>2457</v>
+        <v>2458</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>217</v>
+        <v>316</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>2458</v>
+        <v>2459</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>309</v>
+        <v>217</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>2459</v>
+        <v>2460</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>2460</v>
+        <v>2461</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>2461</v>
+        <v>320</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>2462</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>267</v>
+        <v>2463</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>2463</v>
+        <v>2464</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>329</v>
+        <v>267</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>2464</v>
+        <v>2465</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>221</v>
+        <v>329</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>2465</v>
-      </c>
-      <c r="D142" s="3" t="s">
         <v>2466</v>
+      </c>
+      <c r="C142" s="3" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>2467</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B144" s="3" t="s">
+        <v>2469</v>
+      </c>
+      <c r="D144" s="3" t="s">
         <v>2468</v>
-      </c>
-      <c r="C144" s="3" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>2469</v>
+        <v>2470</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>2470</v>
+        <v>2471</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>2471</v>
+        <v>2472</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>2472</v>
+        <v>2473</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>284</v>
+        <v>249</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>2473</v>
+        <v>2474</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>2474</v>
+        <v>284</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B150" s="3" t="s">
         <v>2475</v>
       </c>
-      <c r="D150" s="3" t="s">
-        <v>2466</v>
+      <c r="C150" s="3" t="s">
+        <v>2476</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>2476</v>
+        <v>2477</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>2466</v>
+        <v>2468</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>2477</v>
-      </c>
-      <c r="C152" s="3" t="s">
-        <v>377</v>
+        <v>2478</v>
+      </c>
+      <c r="D152" s="3" t="s">
+        <v>2468</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>2478</v>
+        <v>2479</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>2479</v>
+        <v>2480</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>2480</v>
+        <v>381</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>2481</v>
@@ -36440,54 +36446,54 @@
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>2483</v>
       </c>
-      <c r="D156" s="3" t="s">
+      <c r="C156" s="3" t="s">
         <v>2484</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>2485</v>
       </c>
-      <c r="C157" s="3" t="s">
+      <c r="D157" s="3" t="s">
         <v>2486</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>2487</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>426</v>
+        <v>2488</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>2488</v>
+        <v>2489</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>454</v>
+        <v>426</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>2489</v>
+        <v>2490</v>
       </c>
       <c r="C160" s="3" t="s">
         <v>454</v>
@@ -36495,18 +36501,18 @@
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>2490</v>
+        <v>2491</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>2491</v>
+        <v>454</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>2492</v>
@@ -36517,7 +36523,7 @@
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>2494</v>
@@ -36528,139 +36534,139 @@
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>2496</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>417</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B165" s="3" t="s">
-        <v>2497</v>
+        <v>2498</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>385</v>
+        <v>417</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B166" s="3" t="s">
-        <v>2498</v>
+        <v>2499</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>434</v>
+        <v>385</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B167" s="3" t="s">
-        <v>2499</v>
+        <v>2500</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>390</v>
+        <v>434</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B168" s="3" t="s">
-        <v>2500</v>
+        <v>2501</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>438</v>
+        <v>390</v>
       </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B169" s="3" t="s">
-        <v>2501</v>
+        <v>2502</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>478</v>
+        <v>438</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B170" s="3" t="s">
-        <v>2502</v>
+        <v>2503</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>441</v>
+        <v>478</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B171" s="3" t="s">
-        <v>2503</v>
+        <v>2504</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>450</v>
+        <v>441</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>2504</v>
+        <v>2505</v>
       </c>
       <c r="C172" s="3" t="s">
-        <v>410</v>
+        <v>450</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B173" s="3" t="s">
-        <v>2505</v>
+        <v>2506</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>393</v>
+        <v>410</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B174" s="3" t="s">
-        <v>2506</v>
+        <v>2507</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>458</v>
+        <v>393</v>
       </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>2507</v>
-      </c>
-      <c r="D175" s="3" t="s">
         <v>2508</v>
+      </c>
+      <c r="C175" s="3" t="s">
+        <v>458</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>2509</v>
@@ -36671,7 +36677,7 @@
     </row>
     <row r="177" spans="1:4">
       <c r="A177" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>2511</v>
@@ -36682,7 +36688,7 @@
     </row>
     <row r="178" spans="1:4">
       <c r="A178" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>2513</v>
@@ -36693,7 +36699,7 @@
     </row>
     <row r="179" spans="1:4">
       <c r="A179" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>2515</v>
@@ -36704,205 +36710,205 @@
     </row>
     <row r="180" spans="1:4">
       <c r="A180" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>2517</v>
       </c>
-      <c r="C180" s="3" t="s">
+      <c r="D180" s="3" t="s">
         <v>2518</v>
       </c>
     </row>
     <row r="181" spans="1:4">
       <c r="A181" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>2519</v>
       </c>
       <c r="C181" s="3" t="s">
-        <v>499</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="182" spans="1:4">
       <c r="A182" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B182" s="3" t="s">
-        <v>2520</v>
+        <v>2521</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>510</v>
+        <v>499</v>
       </c>
     </row>
     <row r="183" spans="1:4">
       <c r="A183" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>2521</v>
+        <v>2522</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>513</v>
+        <v>510</v>
       </c>
     </row>
     <row r="184" spans="1:4">
       <c r="A184" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>2522</v>
+        <v>2523</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
     </row>
     <row r="185" spans="1:4">
       <c r="A185" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>2523</v>
+        <v>2524</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>520</v>
+        <v>517</v>
       </c>
     </row>
     <row r="186" spans="1:4">
       <c r="A186" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>2524</v>
-      </c>
-      <c r="D186" s="3" t="s">
         <v>2525</v>
+      </c>
+      <c r="C186" s="3" t="s">
+        <v>520</v>
       </c>
     </row>
     <row r="187" spans="1:4">
       <c r="A187" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>2526</v>
       </c>
-      <c r="C187" s="3" t="s">
-        <v>524</v>
+      <c r="D187" s="3" t="s">
+        <v>2527</v>
       </c>
     </row>
     <row r="188" spans="1:4">
       <c r="A188" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>2527</v>
+        <v>2528</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>527</v>
+        <v>524</v>
       </c>
     </row>
     <row r="189" spans="1:4">
       <c r="A189" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B189" s="3" t="s">
-        <v>2528</v>
+        <v>2529</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>506</v>
+        <v>527</v>
       </c>
     </row>
     <row r="190" spans="1:4">
       <c r="A190" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B190" s="3" t="s">
-        <v>2529</v>
-      </c>
-      <c r="D190" s="3" t="s">
         <v>2530</v>
+      </c>
+      <c r="C190" s="3" t="s">
+        <v>506</v>
       </c>
     </row>
     <row r="191" spans="1:4">
       <c r="A191" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>2531</v>
       </c>
-      <c r="C191" s="3" t="s">
-        <v>550</v>
+      <c r="D191" s="3" t="s">
+        <v>2532</v>
       </c>
     </row>
     <row r="192" spans="1:4">
       <c r="A192" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B192" s="3" t="s">
-        <v>2532</v>
+        <v>2533</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>554</v>
+        <v>550</v>
       </c>
     </row>
     <row r="193" spans="1:4">
       <c r="A193" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B193" s="3" t="s">
-        <v>2533</v>
+        <v>2534</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>563</v>
+        <v>554</v>
       </c>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B194" s="3" t="s">
-        <v>2534</v>
+        <v>2535</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>567</v>
+        <v>563</v>
       </c>
     </row>
     <row r="195" spans="1:4">
       <c r="A195" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B195" s="3" t="s">
-        <v>2535</v>
+        <v>2536</v>
       </c>
       <c r="C195" s="3" t="s">
-        <v>571</v>
+        <v>567</v>
       </c>
     </row>
     <row r="196" spans="1:4">
       <c r="A196" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B196" s="3" t="s">
-        <v>2536</v>
+        <v>2537</v>
       </c>
       <c r="C196" s="3" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="197" spans="1:4">
       <c r="A197" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B197" s="3" t="s">
-        <v>2537</v>
+        <v>2538</v>
       </c>
       <c r="C197" s="3" t="s">
-        <v>2538</v>
+        <v>574</v>
       </c>
     </row>
     <row r="198" spans="1:4">
       <c r="A198" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>2539</v>
@@ -36913,73 +36919,73 @@
     </row>
     <row r="199" spans="1:4">
       <c r="A199" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>2541</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>589</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="200" spans="1:4">
       <c r="A200" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>2542</v>
+        <v>2543</v>
       </c>
       <c r="C200" s="3" t="s">
-        <v>482</v>
+        <v>589</v>
       </c>
     </row>
     <row r="201" spans="1:4">
       <c r="A201" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B201" s="3" t="s">
-        <v>2543</v>
+        <v>2544</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>495</v>
+        <v>482</v>
       </c>
     </row>
     <row r="202" spans="1:4">
       <c r="A202" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B202" s="3" t="s">
-        <v>2544</v>
+        <v>2545</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B203" s="3" t="s">
-        <v>2545</v>
+        <v>2546</v>
       </c>
       <c r="C203" s="3" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
     </row>
     <row r="204" spans="1:4">
       <c r="A204" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>2546</v>
-      </c>
-      <c r="D204" s="3" t="s">
         <v>2547</v>
+      </c>
+      <c r="C204" s="3" t="s">
+        <v>491</v>
       </c>
     </row>
     <row r="205" spans="1:4">
       <c r="A205" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B205" s="3" t="s">
         <v>2548</v>
@@ -36990,29 +36996,29 @@
     </row>
     <row r="206" spans="1:4">
       <c r="A206" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B206" s="3" t="s">
         <v>2550</v>
       </c>
-      <c r="C206" s="3" t="s">
-        <v>598</v>
+      <c r="D206" s="3" t="s">
+        <v>2551</v>
       </c>
     </row>
     <row r="207" spans="1:4">
       <c r="A207" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B207" s="3" t="s">
-        <v>2551</v>
+        <v>2552</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>2552</v>
+        <v>598</v>
       </c>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B208" s="3" t="s">
         <v>2553</v>
@@ -37023,197 +37029,197 @@
     </row>
     <row r="209" spans="1:3">
       <c r="A209" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B209" s="3" t="s">
         <v>2555</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>615</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>2556</v>
+        <v>2557</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>2557</v>
+        <v>615</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B211" s="3" t="s">
         <v>2558</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>628</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>2559</v>
+        <v>2560</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>620</v>
+        <v>628</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>2560</v>
+        <v>2561</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>636</v>
+        <v>620</v>
       </c>
     </row>
     <row r="214" spans="1:3">
       <c r="A214" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B214" s="3" t="s">
-        <v>2561</v>
+        <v>2562</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
     </row>
     <row r="215" spans="1:3">
       <c r="A215" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>2562</v>
+        <v>2563</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>2563</v>
+        <v>632</v>
       </c>
     </row>
     <row r="216" spans="1:3">
       <c r="A216" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B216" s="3" t="s">
         <v>2564</v>
       </c>
       <c r="C216" s="3" t="s">
-        <v>645</v>
+        <v>2565</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>2565</v>
+        <v>2566</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>676</v>
+        <v>645</v>
       </c>
     </row>
     <row r="218" spans="1:3">
       <c r="A218" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B218" s="3" t="s">
-        <v>2566</v>
+        <v>2567</v>
       </c>
       <c r="C218" s="3" t="s">
-        <v>664</v>
+        <v>676</v>
       </c>
     </row>
     <row r="219" spans="1:3">
       <c r="A219" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>2567</v>
+        <v>2568</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>685</v>
+        <v>664</v>
       </c>
     </row>
     <row r="220" spans="1:3">
       <c r="A220" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B220" s="3" t="s">
-        <v>2568</v>
+        <v>2569</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>673</v>
+        <v>685</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>2569</v>
+        <v>2570</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>654</v>
+        <v>673</v>
       </c>
     </row>
     <row r="222" spans="1:3">
       <c r="A222" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>2570</v>
+        <v>2571</v>
       </c>
       <c r="C222" s="3" t="s">
-        <v>2571</v>
+        <v>654</v>
       </c>
     </row>
     <row r="223" spans="1:3">
       <c r="A223" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B223" s="3" t="s">
         <v>2572</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>692</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B224" s="3" t="s">
-        <v>2573</v>
+        <v>2574</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>639</v>
+        <v>692</v>
       </c>
     </row>
     <row r="225" spans="1:4">
       <c r="A225" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>2574</v>
+        <v>2575</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>650</v>
+        <v>639</v>
       </c>
     </row>
     <row r="226" spans="1:4">
       <c r="A226" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>2575</v>
+        <v>2576</v>
       </c>
       <c r="C226" s="3" t="s">
         <v>650</v>
@@ -37221,24 +37227,24 @@
     </row>
     <row r="227" spans="1:4">
       <c r="A227" s="3" t="s">
-        <v>2396</v>
+        <v>2398</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>2576</v>
+        <v>2577</v>
       </c>
       <c r="C227" s="3" t="s">
-        <v>698</v>
+        <v>650</v>
       </c>
     </row>
     <row r="228" spans="1:4">
       <c r="A228" s="3" t="s">
-        <v>532</v>
+        <v>2398</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>2577</v>
-      </c>
-      <c r="D228" s="3" t="s">
         <v>2578</v>
+      </c>
+      <c r="C228" s="3" t="s">
+        <v>698</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -37271,7 +37277,7 @@
         <v>2583</v>
       </c>
       <c r="D231" s="3" t="s">
-        <v>2578</v>
+        <v>2584</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -37279,10 +37285,10 @@
         <v>532</v>
       </c>
       <c r="B232" s="3" t="s">
-        <v>2584</v>
+        <v>2585</v>
       </c>
       <c r="D232" s="3" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -37290,10 +37296,10 @@
         <v>532</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>2585</v>
+        <v>2586</v>
       </c>
       <c r="D233" s="3" t="s">
-        <v>2578</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -37301,10 +37307,10 @@
         <v>532</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>2586</v>
-      </c>
-      <c r="C234" s="3" t="s">
-        <v>478</v>
+        <v>2587</v>
+      </c>
+      <c r="D234" s="3" t="s">
+        <v>2580</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -37312,10 +37318,10 @@
         <v>532</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>2587</v>
-      </c>
-      <c r="D235" s="3" t="s">
         <v>2588</v>
+      </c>
+      <c r="C235" s="3" t="s">
+        <v>478</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -37417,8 +37423,19 @@
         <v>2606</v>
       </c>
     </row>
+    <row r="245" spans="1:4">
+      <c r="A245" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="B245" s="3" t="s">
+        <v>2607</v>
+      </c>
+      <c r="D245" s="3" t="s">
+        <v>2608</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D244"/>
+  <autoFilter ref="A1:D245"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not in the list" error="Pick one of: operation, job, schedule, handler." promptTitle="Kind" prompt="operation, job, schedule or handler" sqref="A2:A2001">
       <formula1>"operation,job,schedule,handler"</formula1>
@@ -37443,198 +37460,198 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>2607</v>
+        <v>2609</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2608</v>
+        <v>2610</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2609</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>2610</v>
+        <v>2612</v>
       </c>
       <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2611</v>
+        <v>2613</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2612</v>
+        <v>2614</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2614</v>
+        <v>2616</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2615</v>
+        <v>2617</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2616</v>
+        <v>2618</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2617</v>
+        <v>2619</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>2613</v>
+        <v>2615</v>
       </c>
       <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2618</v>
+        <v>2620</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2619</v>
+        <v>2621</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2621</v>
+        <v>2623</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2622</v>
+        <v>2624</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2623</v>
+        <v>2625</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2624</v>
+        <v>2626</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>2625</v>
+        <v>2627</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2626</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2627</v>
+        <v>2629</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2628</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>2629</v>
+        <v>2631</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>2630</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>2631</v>
+        <v>2633</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2632</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>2633</v>
+        <v>2635</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>2634</v>
+        <v>2636</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>2635</v>
+        <v>2637</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>2636</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>2620</v>
+        <v>2622</v>
       </c>
       <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2637</v>
+        <v>2639</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2638</v>
+        <v>2640</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(conversations): track an upload as a draft change; OpenAPI, tracking plan 20 (cloud#391)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -18,8 +18,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Actors!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$282</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$283</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Enums!$A$1:$C$469</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Events!$A$1:$L$169</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Properties!$A$1:$K$358</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8801" uniqueCount="2897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8807" uniqueCount="2901">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -38,7 +38,7 @@
     <t>Plan version</t>
   </si>
   <si>
-    <t>19 (2026-10-27)</t>
+    <t>20 (2026-10-28)</t>
   </si>
   <si>
     <t>What this is</t>
@@ -8102,6 +8102,9 @@
     <t>conversations.rule_updated, conversations.rule_removed</t>
   </si>
   <si>
+    <t>conversations.upload_draft_attachment</t>
+  </si>
+  <si>
     <t>conversations.write_nudge</t>
   </si>
   <si>
@@ -8721,6 +8724,15 @@
   </si>
   <si>
     <t>#685</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>Attaching a file to a draft (campbooks-cloud#391): Coverage for conversations.upload_draft_attachment, which tracks conversations.draft_updated as a save does.</t>
+  </si>
+  <si>
+    <t>#391</t>
   </si>
 </sst>
 </file>
@@ -37657,7 +37669,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D282"/>
+  <dimension ref="A1:D283"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -39502,8 +39514,8 @@
       <c r="B167" s="3" t="s">
         <v>2690</v>
       </c>
-      <c r="D167" s="3" t="s">
-        <v>2681</v>
+      <c r="C167" s="3" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="168" spans="1:4">
@@ -39524,8 +39536,8 @@
       <c r="B169" s="3" t="s">
         <v>2692</v>
       </c>
-      <c r="C169" s="3" t="s">
-        <v>377</v>
+      <c r="D169" s="3" t="s">
+        <v>2681</v>
       </c>
     </row>
     <row r="170" spans="1:4">
@@ -39536,7 +39548,7 @@
         <v>2693</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="171" spans="1:4">
@@ -39547,7 +39559,7 @@
         <v>2694</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>2695</v>
+        <v>381</v>
       </c>
     </row>
     <row r="172" spans="1:4">
@@ -39555,10 +39567,10 @@
         <v>2609</v>
       </c>
       <c r="B172" s="3" t="s">
+        <v>2695</v>
+      </c>
+      <c r="C172" s="3" t="s">
         <v>2696</v>
-      </c>
-      <c r="C172" s="3" t="s">
-        <v>2697</v>
       </c>
     </row>
     <row r="173" spans="1:4">
@@ -39566,10 +39578,10 @@
         <v>2609</v>
       </c>
       <c r="B173" s="3" t="s">
+        <v>2697</v>
+      </c>
+      <c r="C173" s="3" t="s">
         <v>2698</v>
-      </c>
-      <c r="D173" s="3" t="s">
-        <v>2699</v>
       </c>
     </row>
     <row r="174" spans="1:4">
@@ -39577,10 +39589,10 @@
         <v>2609</v>
       </c>
       <c r="B174" s="3" t="s">
+        <v>2699</v>
+      </c>
+      <c r="D174" s="3" t="s">
         <v>2700</v>
-      </c>
-      <c r="C174" s="3" t="s">
-        <v>2701</v>
       </c>
     </row>
     <row r="175" spans="1:4">
@@ -39588,10 +39600,10 @@
         <v>2609</v>
       </c>
       <c r="B175" s="3" t="s">
+        <v>2701</v>
+      </c>
+      <c r="C175" s="3" t="s">
         <v>2702</v>
-      </c>
-      <c r="C175" s="3" t="s">
-        <v>426</v>
       </c>
     </row>
     <row r="176" spans="1:4">
@@ -39602,10 +39614,10 @@
         <v>2703</v>
       </c>
       <c r="C176" s="3" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="177" spans="1:3">
       <c r="A177" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39616,7 +39628,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="178" spans="1:4">
+    <row r="178" spans="1:3">
       <c r="A178" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39624,43 +39636,43 @@
         <v>2705</v>
       </c>
       <c r="C178" s="3" t="s">
-        <v>2706</v>
-      </c>
-    </row>
-    <row r="179" spans="1:4">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3">
       <c r="A179" s="3" t="s">
         <v>2609</v>
       </c>
       <c r="B179" s="3" t="s">
+        <v>2706</v>
+      </c>
+      <c r="C179" s="3" t="s">
         <v>2707</v>
       </c>
-      <c r="C179" s="3" t="s">
-        <v>2708</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4">
+    </row>
+    <row r="180" spans="1:3">
       <c r="A180" s="3" t="s">
         <v>2609</v>
       </c>
       <c r="B180" s="3" t="s">
+        <v>2708</v>
+      </c>
+      <c r="C180" s="3" t="s">
         <v>2709</v>
       </c>
-      <c r="C180" s="3" t="s">
-        <v>2710</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4">
+    </row>
+    <row r="181" spans="1:3">
       <c r="A181" s="3" t="s">
         <v>2609</v>
       </c>
       <c r="B181" s="3" t="s">
+        <v>2710</v>
+      </c>
+      <c r="C181" s="3" t="s">
         <v>2711</v>
       </c>
-      <c r="C181" s="3" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4">
+    </row>
+    <row r="182" spans="1:3">
       <c r="A182" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39668,10 +39680,10 @@
         <v>2712</v>
       </c>
       <c r="C182" s="3" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="183" spans="1:3">
       <c r="A183" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39679,10 +39691,10 @@
         <v>2713</v>
       </c>
       <c r="C183" s="3" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="184" spans="1:3">
       <c r="A184" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39690,10 +39702,10 @@
         <v>2714</v>
       </c>
       <c r="C184" s="3" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="185" spans="1:4">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="185" spans="1:3">
       <c r="A185" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39701,10 +39713,10 @@
         <v>2715</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="186" spans="1:4">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="186" spans="1:3">
       <c r="A186" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39712,10 +39724,10 @@
         <v>2716</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3">
       <c r="A187" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39723,10 +39735,10 @@
         <v>2717</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="188" spans="1:3">
       <c r="A188" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39734,10 +39746,10 @@
         <v>2718</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="189" spans="1:3">
       <c r="A189" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39745,10 +39757,10 @@
         <v>2719</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="190" spans="1:4">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="190" spans="1:3">
       <c r="A190" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39756,10 +39768,10 @@
         <v>2720</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>393</v>
-      </c>
-    </row>
-    <row r="191" spans="1:4">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3">
       <c r="A191" s="3" t="s">
         <v>2609</v>
       </c>
@@ -39767,18 +39779,18 @@
         <v>2721</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="192" spans="1:4">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="192" spans="1:3">
       <c r="A192" s="3" t="s">
         <v>2609</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>2722</v>
       </c>
-      <c r="D192" s="3" t="s">
-        <v>2723</v>
+      <c r="C192" s="3" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="193" spans="1:4">
@@ -39786,10 +39798,10 @@
         <v>2609</v>
       </c>
       <c r="B193" s="3" t="s">
+        <v>2723</v>
+      </c>
+      <c r="D193" s="3" t="s">
         <v>2724</v>
-      </c>
-      <c r="D193" s="3" t="s">
-        <v>2725</v>
       </c>
     </row>
     <row r="194" spans="1:4">
@@ -39797,10 +39809,10 @@
         <v>2609</v>
       </c>
       <c r="B194" s="3" t="s">
+        <v>2725</v>
+      </c>
+      <c r="D194" s="3" t="s">
         <v>2726</v>
-      </c>
-      <c r="D194" s="3" t="s">
-        <v>2727</v>
       </c>
     </row>
     <row r="195" spans="1:4">
@@ -39808,10 +39820,10 @@
         <v>2609</v>
       </c>
       <c r="B195" s="3" t="s">
+        <v>2727</v>
+      </c>
+      <c r="D195" s="3" t="s">
         <v>2728</v>
-      </c>
-      <c r="D195" s="3" t="s">
-        <v>2729</v>
       </c>
     </row>
     <row r="196" spans="1:4">
@@ -39819,10 +39831,10 @@
         <v>2609</v>
       </c>
       <c r="B196" s="3" t="s">
+        <v>2729</v>
+      </c>
+      <c r="D196" s="3" t="s">
         <v>2730</v>
-      </c>
-      <c r="D196" s="3" t="s">
-        <v>2731</v>
       </c>
     </row>
     <row r="197" spans="1:4">
@@ -39830,10 +39842,10 @@
         <v>2609</v>
       </c>
       <c r="B197" s="3" t="s">
+        <v>2731</v>
+      </c>
+      <c r="D197" s="3" t="s">
         <v>2732</v>
-      </c>
-      <c r="C197" s="3" t="s">
-        <v>2733</v>
       </c>
     </row>
     <row r="198" spans="1:4">
@@ -39841,10 +39853,10 @@
         <v>2609</v>
       </c>
       <c r="B198" s="3" t="s">
+        <v>2733</v>
+      </c>
+      <c r="C198" s="3" t="s">
         <v>2734</v>
-      </c>
-      <c r="C198" s="3" t="s">
-        <v>586</v>
       </c>
     </row>
     <row r="199" spans="1:4">
@@ -39855,7 +39867,7 @@
         <v>2735</v>
       </c>
       <c r="C199" s="3" t="s">
-        <v>2736</v>
+        <v>586</v>
       </c>
     </row>
     <row r="200" spans="1:4">
@@ -39863,10 +39875,10 @@
         <v>2609</v>
       </c>
       <c r="B200" s="3" t="s">
+        <v>2736</v>
+      </c>
+      <c r="C200" s="3" t="s">
         <v>2737</v>
-      </c>
-      <c r="C200" s="3" t="s">
-        <v>556</v>
       </c>
     </row>
     <row r="201" spans="1:4">
@@ -39877,7 +39889,7 @@
         <v>2738</v>
       </c>
       <c r="C201" s="3" t="s">
-        <v>2739</v>
+        <v>556</v>
       </c>
     </row>
     <row r="202" spans="1:4">
@@ -39885,10 +39897,10 @@
         <v>2609</v>
       </c>
       <c r="B202" s="3" t="s">
+        <v>2739</v>
+      </c>
+      <c r="C202" s="3" t="s">
         <v>2740</v>
-      </c>
-      <c r="C202" s="3" t="s">
-        <v>599</v>
       </c>
     </row>
     <row r="203" spans="1:4">
@@ -39898,8 +39910,8 @@
       <c r="B203" s="3" t="s">
         <v>2741</v>
       </c>
-      <c r="D203" s="3" t="s">
-        <v>2742</v>
+      <c r="C203" s="3" t="s">
+        <v>599</v>
       </c>
     </row>
     <row r="204" spans="1:4">
@@ -39907,10 +39919,10 @@
         <v>2609</v>
       </c>
       <c r="B204" s="3" t="s">
+        <v>2742</v>
+      </c>
+      <c r="D204" s="3" t="s">
         <v>2743</v>
-      </c>
-      <c r="C204" s="3" t="s">
-        <v>2744</v>
       </c>
     </row>
     <row r="205" spans="1:4">
@@ -39918,10 +39930,10 @@
         <v>2609</v>
       </c>
       <c r="B205" s="3" t="s">
+        <v>2744</v>
+      </c>
+      <c r="C205" s="3" t="s">
         <v>2745</v>
-      </c>
-      <c r="C205" s="3" t="s">
-        <v>565</v>
       </c>
     </row>
     <row r="206" spans="1:4">
@@ -39932,7 +39944,7 @@
         <v>2746</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>568</v>
+        <v>565</v>
       </c>
     </row>
     <row r="207" spans="1:4">
@@ -39943,7 +39955,7 @@
         <v>2747</v>
       </c>
       <c r="C207" s="3" t="s">
-        <v>590</v>
+        <v>568</v>
       </c>
     </row>
     <row r="208" spans="1:4">
@@ -39953,8 +39965,8 @@
       <c r="B208" s="3" t="s">
         <v>2748</v>
       </c>
-      <c r="D208" s="3" t="s">
-        <v>2749</v>
+      <c r="C208" s="3" t="s">
+        <v>590</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -39962,10 +39974,10 @@
         <v>2609</v>
       </c>
       <c r="B209" s="3" t="s">
+        <v>2749</v>
+      </c>
+      <c r="D209" s="3" t="s">
         <v>2750</v>
-      </c>
-      <c r="D209" s="3" t="s">
-        <v>2751</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -39973,10 +39985,10 @@
         <v>2609</v>
       </c>
       <c r="B210" s="3" t="s">
+        <v>2751</v>
+      </c>
+      <c r="D210" s="3" t="s">
         <v>2752</v>
-      </c>
-      <c r="C210" s="3" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -39987,7 +39999,7 @@
         <v>2753</v>
       </c>
       <c r="C211" s="3" t="s">
-        <v>549</v>
+        <v>524</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -39998,7 +40010,7 @@
         <v>2754</v>
       </c>
       <c r="C212" s="3" t="s">
-        <v>572</v>
+        <v>549</v>
       </c>
     </row>
     <row r="213" spans="1:4">
@@ -40008,8 +40020,8 @@
       <c r="B213" s="3" t="s">
         <v>2755</v>
       </c>
-      <c r="D213" s="3" t="s">
-        <v>2756</v>
+      <c r="C213" s="3" t="s">
+        <v>572</v>
       </c>
     </row>
     <row r="214" spans="1:4">
@@ -40017,10 +40029,10 @@
         <v>2609</v>
       </c>
       <c r="B214" s="3" t="s">
+        <v>2756</v>
+      </c>
+      <c r="D214" s="3" t="s">
         <v>2757</v>
-      </c>
-      <c r="C214" s="3" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -40030,8 +40042,8 @@
       <c r="B215" s="3" t="s">
         <v>2758</v>
       </c>
-      <c r="D215" s="3" t="s">
-        <v>2759</v>
+      <c r="C215" s="3" t="s">
+        <v>511</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -40039,10 +40051,10 @@
         <v>2609</v>
       </c>
       <c r="B216" s="3" t="s">
+        <v>2759</v>
+      </c>
+      <c r="D216" s="3" t="s">
         <v>2760</v>
-      </c>
-      <c r="C216" s="3" t="s">
-        <v>575</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -40053,7 +40065,7 @@
         <v>2761</v>
       </c>
       <c r="C217" s="3" t="s">
-        <v>541</v>
+        <v>575</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -40074,8 +40086,8 @@
       <c r="B219" s="3" t="s">
         <v>2763</v>
       </c>
-      <c r="D219" s="3" t="s">
-        <v>2764</v>
+      <c r="C219" s="3" t="s">
+        <v>541</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -40083,10 +40095,10 @@
         <v>2609</v>
       </c>
       <c r="B220" s="3" t="s">
+        <v>2764</v>
+      </c>
+      <c r="D220" s="3" t="s">
         <v>2765</v>
-      </c>
-      <c r="C220" s="3" t="s">
-        <v>579</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -40097,7 +40109,7 @@
         <v>2766</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>518</v>
+        <v>579</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -40108,7 +40120,7 @@
         <v>2767</v>
       </c>
       <c r="C222" s="3" t="s">
-        <v>545</v>
+        <v>518</v>
       </c>
     </row>
     <row r="223" spans="1:4">
@@ -40119,7 +40131,7 @@
         <v>2768</v>
       </c>
       <c r="C223" s="3" t="s">
-        <v>582</v>
+        <v>545</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -40130,7 +40142,7 @@
         <v>2769</v>
       </c>
       <c r="C224" s="3" t="s">
-        <v>562</v>
+        <v>582</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -40140,8 +40152,8 @@
       <c r="B225" s="3" t="s">
         <v>2770</v>
       </c>
-      <c r="D225" s="3" t="s">
-        <v>2771</v>
+      <c r="C225" s="3" t="s">
+        <v>562</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -40149,10 +40161,10 @@
         <v>2609</v>
       </c>
       <c r="B226" s="3" t="s">
+        <v>2771</v>
+      </c>
+      <c r="D226" s="3" t="s">
         <v>2772</v>
-      </c>
-      <c r="D226" s="3" t="s">
-        <v>2773</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -40160,10 +40172,10 @@
         <v>2609</v>
       </c>
       <c r="B227" s="3" t="s">
+        <v>2773</v>
+      </c>
+      <c r="D227" s="3" t="s">
         <v>2774</v>
-      </c>
-      <c r="D227" s="3" t="s">
-        <v>2775</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -40171,10 +40183,10 @@
         <v>2609</v>
       </c>
       <c r="B228" s="3" t="s">
+        <v>2775</v>
+      </c>
+      <c r="D228" s="3" t="s">
         <v>2776</v>
-      </c>
-      <c r="C228" s="3" t="s">
-        <v>622</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -40185,7 +40197,7 @@
         <v>2777</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>626</v>
+        <v>622</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -40196,7 +40208,7 @@
         <v>2778</v>
       </c>
       <c r="C230" s="3" t="s">
-        <v>635</v>
+        <v>626</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -40207,7 +40219,7 @@
         <v>2779</v>
       </c>
       <c r="C231" s="3" t="s">
-        <v>639</v>
+        <v>635</v>
       </c>
     </row>
     <row r="232" spans="1:4">
@@ -40218,7 +40230,7 @@
         <v>2780</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>643</v>
+        <v>639</v>
       </c>
     </row>
     <row r="233" spans="1:4">
@@ -40229,7 +40241,7 @@
         <v>2781</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>646</v>
+        <v>643</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -40240,7 +40252,7 @@
         <v>2782</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>2783</v>
+        <v>646</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -40248,10 +40260,10 @@
         <v>2609</v>
       </c>
       <c r="B235" s="3" t="s">
+        <v>2783</v>
+      </c>
+      <c r="C235" s="3" t="s">
         <v>2784</v>
-      </c>
-      <c r="C235" s="3" t="s">
-        <v>2785</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -40259,10 +40271,10 @@
         <v>2609</v>
       </c>
       <c r="B236" s="3" t="s">
+        <v>2785</v>
+      </c>
+      <c r="C236" s="3" t="s">
         <v>2786</v>
-      </c>
-      <c r="C236" s="3" t="s">
-        <v>661</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -40273,7 +40285,7 @@
         <v>2787</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>494</v>
+        <v>661</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -40284,7 +40296,7 @@
         <v>2788</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -40295,7 +40307,7 @@
         <v>2789</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -40306,7 +40318,7 @@
         <v>2790</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
     </row>
     <row r="241" spans="1:4">
@@ -40316,8 +40328,8 @@
       <c r="B241" s="3" t="s">
         <v>2791</v>
       </c>
-      <c r="D241" s="3" t="s">
-        <v>2792</v>
+      <c r="C241" s="3" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -40325,10 +40337,10 @@
         <v>2609</v>
       </c>
       <c r="B242" s="3" t="s">
+        <v>2792</v>
+      </c>
+      <c r="D242" s="3" t="s">
         <v>2793</v>
-      </c>
-      <c r="D242" s="3" t="s">
-        <v>2794</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -40336,10 +40348,10 @@
         <v>2609</v>
       </c>
       <c r="B243" s="3" t="s">
+        <v>2794</v>
+      </c>
+      <c r="D243" s="3" t="s">
         <v>2795</v>
-      </c>
-      <c r="C243" s="3" t="s">
-        <v>670</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -40350,7 +40362,7 @@
         <v>2796</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>2797</v>
+        <v>670</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -40358,10 +40370,10 @@
         <v>2609</v>
       </c>
       <c r="B245" s="3" t="s">
+        <v>2797</v>
+      </c>
+      <c r="C245" s="3" t="s">
         <v>2798</v>
-      </c>
-      <c r="C245" s="3" t="s">
-        <v>2799</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -40369,10 +40381,10 @@
         <v>2609</v>
       </c>
       <c r="B246" s="3" t="s">
+        <v>2799</v>
+      </c>
+      <c r="C246" s="3" t="s">
         <v>2800</v>
-      </c>
-      <c r="C246" s="3" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -40383,7 +40395,7 @@
         <v>2801</v>
       </c>
       <c r="C247" s="3" t="s">
-        <v>2802</v>
+        <v>687</v>
       </c>
     </row>
     <row r="248" spans="1:4">
@@ -40391,10 +40403,10 @@
         <v>2609</v>
       </c>
       <c r="B248" s="3" t="s">
+        <v>2802</v>
+      </c>
+      <c r="C248" s="3" t="s">
         <v>2803</v>
-      </c>
-      <c r="C248" s="3" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -40405,7 +40417,7 @@
         <v>2804</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>692</v>
+        <v>700</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -40416,7 +40428,7 @@
         <v>2805</v>
       </c>
       <c r="C250" s="3" t="s">
-        <v>708</v>
+        <v>692</v>
       </c>
     </row>
     <row r="251" spans="1:4">
@@ -40427,7 +40439,7 @@
         <v>2806</v>
       </c>
       <c r="C251" s="3" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -40438,7 +40450,7 @@
         <v>2807</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>2808</v>
+        <v>704</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -40446,10 +40458,10 @@
         <v>2609</v>
       </c>
       <c r="B253" s="3" t="s">
+        <v>2808</v>
+      </c>
+      <c r="C253" s="3" t="s">
         <v>2809</v>
-      </c>
-      <c r="C253" s="3" t="s">
-        <v>717</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -40460,7 +40472,7 @@
         <v>2810</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>748</v>
+        <v>717</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -40471,7 +40483,7 @@
         <v>2811</v>
       </c>
       <c r="C255" s="3" t="s">
-        <v>736</v>
+        <v>748</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -40482,7 +40494,7 @@
         <v>2812</v>
       </c>
       <c r="C256" s="3" t="s">
-        <v>757</v>
+        <v>736</v>
       </c>
     </row>
     <row r="257" spans="1:4">
@@ -40493,7 +40505,7 @@
         <v>2813</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>745</v>
+        <v>757</v>
       </c>
     </row>
     <row r="258" spans="1:4">
@@ -40504,7 +40516,7 @@
         <v>2814</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>726</v>
+        <v>745</v>
       </c>
     </row>
     <row r="259" spans="1:4">
@@ -40515,7 +40527,7 @@
         <v>2815</v>
       </c>
       <c r="C259" s="3" t="s">
-        <v>2816</v>
+        <v>726</v>
       </c>
     </row>
     <row r="260" spans="1:4">
@@ -40523,10 +40535,10 @@
         <v>2609</v>
       </c>
       <c r="B260" s="3" t="s">
+        <v>2816</v>
+      </c>
+      <c r="C260" s="3" t="s">
         <v>2817</v>
-      </c>
-      <c r="C260" s="3" t="s">
-        <v>764</v>
       </c>
     </row>
     <row r="261" spans="1:4">
@@ -40537,7 +40549,7 @@
         <v>2818</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>711</v>
+        <v>764</v>
       </c>
     </row>
     <row r="262" spans="1:4">
@@ -40548,7 +40560,7 @@
         <v>2819</v>
       </c>
       <c r="C262" s="3" t="s">
-        <v>722</v>
+        <v>711</v>
       </c>
     </row>
     <row r="263" spans="1:4">
@@ -40570,18 +40582,18 @@
         <v>2821</v>
       </c>
       <c r="C264" s="3" t="s">
-        <v>770</v>
+        <v>722</v>
       </c>
     </row>
     <row r="265" spans="1:4">
       <c r="A265" s="3" t="s">
-        <v>604</v>
+        <v>2609</v>
       </c>
       <c r="B265" s="3" t="s">
         <v>2822</v>
       </c>
-      <c r="D265" s="3" t="s">
-        <v>2823</v>
+      <c r="C265" s="3" t="s">
+        <v>770</v>
       </c>
     </row>
     <row r="266" spans="1:4">
@@ -40589,10 +40601,10 @@
         <v>604</v>
       </c>
       <c r="B266" s="3" t="s">
+        <v>2823</v>
+      </c>
+      <c r="D266" s="3" t="s">
         <v>2824</v>
-      </c>
-      <c r="D266" s="3" t="s">
-        <v>2825</v>
       </c>
     </row>
     <row r="267" spans="1:4">
@@ -40600,10 +40612,10 @@
         <v>604</v>
       </c>
       <c r="B267" s="3" t="s">
+        <v>2825</v>
+      </c>
+      <c r="D267" s="3" t="s">
         <v>2826</v>
-      </c>
-      <c r="D267" s="3" t="s">
-        <v>2827</v>
       </c>
     </row>
     <row r="268" spans="1:4">
@@ -40611,10 +40623,10 @@
         <v>604</v>
       </c>
       <c r="B268" s="3" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D268" s="3" t="s">
         <v>2828</v>
-      </c>
-      <c r="D268" s="3" t="s">
-        <v>2823</v>
       </c>
     </row>
     <row r="269" spans="1:4">
@@ -40625,7 +40637,7 @@
         <v>2829</v>
       </c>
       <c r="D269" s="3" t="s">
-        <v>2823</v>
+        <v>2824</v>
       </c>
     </row>
     <row r="270" spans="1:4">
@@ -40636,7 +40648,7 @@
         <v>2830</v>
       </c>
       <c r="D270" s="3" t="s">
-        <v>2823</v>
+        <v>2824</v>
       </c>
     </row>
     <row r="271" spans="1:4">
@@ -40646,8 +40658,8 @@
       <c r="B271" s="3" t="s">
         <v>2831</v>
       </c>
-      <c r="C271" s="3" t="s">
-        <v>490</v>
+      <c r="D271" s="3" t="s">
+        <v>2824</v>
       </c>
     </row>
     <row r="272" spans="1:4">
@@ -40657,8 +40669,8 @@
       <c r="B272" s="3" t="s">
         <v>2832</v>
       </c>
-      <c r="D272" s="3" t="s">
-        <v>2833</v>
+      <c r="C272" s="3" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="273" spans="1:4">
@@ -40666,10 +40678,10 @@
         <v>604</v>
       </c>
       <c r="B273" s="3" t="s">
+        <v>2833</v>
+      </c>
+      <c r="D273" s="3" t="s">
         <v>2834</v>
-      </c>
-      <c r="D273" s="3" t="s">
-        <v>2835</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -40677,10 +40689,10 @@
         <v>604</v>
       </c>
       <c r="B274" s="3" t="s">
+        <v>2835</v>
+      </c>
+      <c r="D274" s="3" t="s">
         <v>2836</v>
-      </c>
-      <c r="D274" s="3" t="s">
-        <v>2837</v>
       </c>
     </row>
     <row r="275" spans="1:4">
@@ -40688,10 +40700,10 @@
         <v>604</v>
       </c>
       <c r="B275" s="3" t="s">
+        <v>2837</v>
+      </c>
+      <c r="D275" s="3" t="s">
         <v>2838</v>
-      </c>
-      <c r="D275" s="3" t="s">
-        <v>2839</v>
       </c>
     </row>
     <row r="276" spans="1:4">
@@ -40699,10 +40711,10 @@
         <v>604</v>
       </c>
       <c r="B276" s="3" t="s">
+        <v>2839</v>
+      </c>
+      <c r="D276" s="3" t="s">
         <v>2840</v>
-      </c>
-      <c r="D276" s="3" t="s">
-        <v>2841</v>
       </c>
     </row>
     <row r="277" spans="1:4">
@@ -40710,10 +40722,10 @@
         <v>604</v>
       </c>
       <c r="B277" s="3" t="s">
+        <v>2841</v>
+      </c>
+      <c r="D277" s="3" t="s">
         <v>2842</v>
-      </c>
-      <c r="D277" s="3" t="s">
-        <v>2843</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -40721,10 +40733,10 @@
         <v>604</v>
       </c>
       <c r="B278" s="3" t="s">
+        <v>2843</v>
+      </c>
+      <c r="D278" s="3" t="s">
         <v>2844</v>
-      </c>
-      <c r="D278" s="3" t="s">
-        <v>2845</v>
       </c>
     </row>
     <row r="279" spans="1:4">
@@ -40732,10 +40744,10 @@
         <v>604</v>
       </c>
       <c r="B279" s="3" t="s">
+        <v>2845</v>
+      </c>
+      <c r="D279" s="3" t="s">
         <v>2846</v>
-      </c>
-      <c r="D279" s="3" t="s">
-        <v>2847</v>
       </c>
     </row>
     <row r="280" spans="1:4">
@@ -40743,10 +40755,10 @@
         <v>604</v>
       </c>
       <c r="B280" s="3" t="s">
+        <v>2847</v>
+      </c>
+      <c r="D280" s="3" t="s">
         <v>2848</v>
-      </c>
-      <c r="D280" s="3" t="s">
-        <v>2849</v>
       </c>
     </row>
     <row r="281" spans="1:4">
@@ -40754,10 +40766,10 @@
         <v>604</v>
       </c>
       <c r="B281" s="3" t="s">
+        <v>2849</v>
+      </c>
+      <c r="D281" s="3" t="s">
         <v>2850</v>
-      </c>
-      <c r="D281" s="3" t="s">
-        <v>2851</v>
       </c>
     </row>
     <row r="282" spans="1:4">
@@ -40765,14 +40777,25 @@
         <v>604</v>
       </c>
       <c r="B282" s="3" t="s">
+        <v>2851</v>
+      </c>
+      <c r="D282" s="3" t="s">
         <v>2852</v>
       </c>
-      <c r="D282" s="3" t="s">
-        <v>2823</v>
+    </row>
+    <row r="283" spans="1:4">
+      <c r="A283" s="3" t="s">
+        <v>604</v>
+      </c>
+      <c r="B283" s="3" t="s">
+        <v>2853</v>
+      </c>
+      <c r="D283" s="3" t="s">
+        <v>2824</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D282"/>
+  <autoFilter ref="A1:D283"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not in the list" error="Pick one of: operation, job, schedule, handler." promptTitle="Kind" prompt="operation, job, schedule or handler" sqref="A2:A2001">
       <formula1>"operation,job,schedule,handler"</formula1>
@@ -40787,7 +40810,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12.7109375" customWidth="1"/>
@@ -40797,272 +40820,286 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>2853</v>
+        <v>2854</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2854</v>
+        <v>2855</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2855</v>
+        <v>2856</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>2856</v>
+        <v>2857</v>
       </c>
       <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2857</v>
+        <v>2858</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2858</v>
+        <v>2859</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>2859</v>
+        <v>2860</v>
       </c>
       <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2860</v>
+        <v>2861</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2861</v>
+        <v>2862</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>2859</v>
+        <v>2860</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2862</v>
+        <v>2863</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2863</v>
+        <v>2864</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>2859</v>
+        <v>2860</v>
       </c>
       <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2864</v>
+        <v>2865</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2865</v>
+        <v>2866</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2867</v>
+        <v>2868</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2868</v>
+        <v>2869</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2869</v>
+        <v>2870</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2870</v>
+        <v>2871</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>2871</v>
+        <v>2872</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2872</v>
+        <v>2873</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2873</v>
+        <v>2874</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2874</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>2875</v>
+        <v>2876</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>2876</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>2877</v>
+        <v>2878</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2878</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>2879</v>
+        <v>2880</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>2880</v>
+        <v>2881</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>2881</v>
+        <v>2882</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2883</v>
+        <v>2884</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2884</v>
+        <v>2885</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="3" t="s">
-        <v>2866</v>
+        <v>2867</v>
       </c>
       <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2885</v>
+        <v>2886</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2886</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="3" t="s">
-        <v>2887</v>
+        <v>2888</v>
       </c>
       <c r="B16" s="3">
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>2888</v>
+        <v>2889</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>2889</v>
+        <v>2890</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="3" t="s">
-        <v>2887</v>
+        <v>2888</v>
       </c>
       <c r="B17" s="3">
         <v>17</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2890</v>
+        <v>2891</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2891</v>
+        <v>2892</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="3" t="s">
-        <v>2887</v>
+        <v>2888</v>
       </c>
       <c r="B18" s="3">
         <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>2892</v>
+        <v>2893</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2893</v>
+        <v>2894</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="3" t="s">
-        <v>2894</v>
+        <v>2895</v>
       </c>
       <c r="B19" s="3">
         <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>2895</v>
+        <v>2896</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>2896</v>
+        <v>2897</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
+      <c r="A20" s="3" t="s">
+        <v>2898</v>
+      </c>
+      <c r="B20" s="3">
+        <v>20</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>2899</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>2900</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D19"/>
+  <autoFilter ref="A1:D20"/>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="YYYY-MM-DD" sqref="A2:A2001"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Plan version" prompt="From 1, one per change." sqref="B2:B2001"/>

</xml_diff>

<commit_message>
fix(pages,assistant,search): security review of #690 (cloud #364)
attach_from_message also needs the conversations:read scope and answers 404 for bytes the store lacks; the Markdown reader is linear in its input (bracket and parenthesis pairs found in one pass, step-counted test); search takes a types limit so find_pages is not crowded out by mail; page proposals carry who can read the target (effective grants, new pages inherit them) and whether Notion keeps a copy, through the new pages.get_sharing; unappend keeps the record while edited blocks remain; the blocks count leaves out the sources line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Actors!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$287</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$288</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Enums!$A$1:$C$473</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Events!$A$1:$L$171</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Properties!$A$1:$K$363</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8890" uniqueCount="2929">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8893" uniqueCount="2931">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -8328,6 +8328,12 @@
   </si>
   <si>
     <t>takes back files that pages.attach_from_message made files of the page, for the ones no block names; nothing new is made, and the files were tracked when they were attached (pages.files_attached)</t>
+  </si>
+  <si>
+    <t>pages.get_sharing</t>
+  </si>
+  <si>
+    <t>reads who can read a page and whether Notion keeps a copy, for Scout's card; it changes nothing</t>
   </si>
   <si>
     <t>pages.get_table_sync</t>
@@ -38015,7 +38021,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D287"/>
+  <dimension ref="A1:D288"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -40300,7 +40306,7 @@
       <c r="B207" s="3" t="s">
         <v>2768</v>
       </c>
-      <c r="C207" s="3" t="s">
+      <c r="D207" s="3" t="s">
         <v>2769</v>
       </c>
     </row>
@@ -40312,7 +40318,7 @@
         <v>2770</v>
       </c>
       <c r="C208" s="3" t="s">
-        <v>571</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="209" spans="1:4">
@@ -40320,10 +40326,10 @@
         <v>2630</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>2771</v>
+        <v>2772</v>
       </c>
       <c r="C209" s="3" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="210" spans="1:4">
@@ -40331,10 +40337,10 @@
         <v>2630</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>2772</v>
+        <v>2773</v>
       </c>
       <c r="C210" s="3" t="s">
-        <v>596</v>
+        <v>574</v>
       </c>
     </row>
     <row r="211" spans="1:4">
@@ -40342,10 +40348,10 @@
         <v>2630</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>2773</v>
-      </c>
-      <c r="D211" s="3" t="s">
         <v>2774</v>
+      </c>
+      <c r="C211" s="3" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="212" spans="1:4">
@@ -40377,8 +40383,8 @@
       <c r="B214" s="3" t="s">
         <v>2779</v>
       </c>
-      <c r="C214" s="3" t="s">
-        <v>530</v>
+      <c r="D214" s="3" t="s">
+        <v>2780</v>
       </c>
     </row>
     <row r="215" spans="1:4">
@@ -40386,10 +40392,10 @@
         <v>2630</v>
       </c>
       <c r="B215" s="3" t="s">
-        <v>2780</v>
+        <v>2781</v>
       </c>
       <c r="C215" s="3" t="s">
-        <v>555</v>
+        <v>530</v>
       </c>
     </row>
     <row r="216" spans="1:4">
@@ -40397,10 +40403,10 @@
         <v>2630</v>
       </c>
       <c r="B216" s="3" t="s">
-        <v>2781</v>
+        <v>2782</v>
       </c>
       <c r="C216" s="3" t="s">
-        <v>578</v>
+        <v>555</v>
       </c>
     </row>
     <row r="217" spans="1:4">
@@ -40408,10 +40414,10 @@
         <v>2630</v>
       </c>
       <c r="B217" s="3" t="s">
-        <v>2782</v>
-      </c>
-      <c r="D217" s="3" t="s">
         <v>2783</v>
+      </c>
+      <c r="C217" s="3" t="s">
+        <v>578</v>
       </c>
     </row>
     <row r="218" spans="1:4">
@@ -40421,8 +40427,8 @@
       <c r="B218" s="3" t="s">
         <v>2784</v>
       </c>
-      <c r="C218" s="3" t="s">
-        <v>511</v>
+      <c r="D218" s="3" t="s">
+        <v>2785</v>
       </c>
     </row>
     <row r="219" spans="1:4">
@@ -40430,10 +40436,10 @@
         <v>2630</v>
       </c>
       <c r="B219" s="3" t="s">
-        <v>2785</v>
-      </c>
-      <c r="D219" s="3" t="s">
         <v>2786</v>
+      </c>
+      <c r="C219" s="3" t="s">
+        <v>511</v>
       </c>
     </row>
     <row r="220" spans="1:4">
@@ -40443,8 +40449,8 @@
       <c r="B220" s="3" t="s">
         <v>2787</v>
       </c>
-      <c r="C220" s="3" t="s">
-        <v>581</v>
+      <c r="D220" s="3" t="s">
+        <v>2788</v>
       </c>
     </row>
     <row r="221" spans="1:4">
@@ -40452,10 +40458,10 @@
         <v>2630</v>
       </c>
       <c r="B221" s="3" t="s">
-        <v>2788</v>
+        <v>2789</v>
       </c>
       <c r="C221" s="3" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="222" spans="1:4">
@@ -40463,7 +40469,7 @@
         <v>2630</v>
       </c>
       <c r="B222" s="3" t="s">
-        <v>2789</v>
+        <v>2790</v>
       </c>
       <c r="C222" s="3" t="s">
         <v>547</v>
@@ -40474,10 +40480,10 @@
         <v>2630</v>
       </c>
       <c r="B223" s="3" t="s">
-        <v>2790</v>
-      </c>
-      <c r="D223" s="3" t="s">
         <v>2791</v>
+      </c>
+      <c r="C223" s="3" t="s">
+        <v>547</v>
       </c>
     </row>
     <row r="224" spans="1:4">
@@ -40487,8 +40493,8 @@
       <c r="B224" s="3" t="s">
         <v>2792</v>
       </c>
-      <c r="C224" s="3" t="s">
-        <v>585</v>
+      <c r="D224" s="3" t="s">
+        <v>2793</v>
       </c>
     </row>
     <row r="225" spans="1:4">
@@ -40496,10 +40502,10 @@
         <v>2630</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>2793</v>
-      </c>
-      <c r="D225" s="3" t="s">
         <v>2794</v>
+      </c>
+      <c r="C225" s="3" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="226" spans="1:4">
@@ -40509,8 +40515,8 @@
       <c r="B226" s="3" t="s">
         <v>2795</v>
       </c>
-      <c r="C226" s="3" t="s">
-        <v>524</v>
+      <c r="D226" s="3" t="s">
+        <v>2796</v>
       </c>
     </row>
     <row r="227" spans="1:4">
@@ -40518,10 +40524,10 @@
         <v>2630</v>
       </c>
       <c r="B227" s="3" t="s">
-        <v>2796</v>
+        <v>2797</v>
       </c>
       <c r="C227" s="3" t="s">
-        <v>551</v>
+        <v>524</v>
       </c>
     </row>
     <row r="228" spans="1:4">
@@ -40529,10 +40535,10 @@
         <v>2630</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>2797</v>
+        <v>2798</v>
       </c>
       <c r="C228" s="3" t="s">
-        <v>588</v>
+        <v>551</v>
       </c>
     </row>
     <row r="229" spans="1:4">
@@ -40540,10 +40546,10 @@
         <v>2630</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>2798</v>
+        <v>2799</v>
       </c>
       <c r="C229" s="3" t="s">
-        <v>568</v>
+        <v>588</v>
       </c>
     </row>
     <row r="230" spans="1:4">
@@ -40551,10 +40557,10 @@
         <v>2630</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>2799</v>
-      </c>
-      <c r="D230" s="3" t="s">
         <v>2800</v>
+      </c>
+      <c r="C230" s="3" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="231" spans="1:4">
@@ -40586,8 +40592,8 @@
       <c r="B233" s="3" t="s">
         <v>2805</v>
       </c>
-      <c r="C233" s="3" t="s">
-        <v>633</v>
+      <c r="D233" s="3" t="s">
+        <v>2806</v>
       </c>
     </row>
     <row r="234" spans="1:4">
@@ -40595,10 +40601,10 @@
         <v>2630</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>2806</v>
+        <v>2807</v>
       </c>
       <c r="C234" s="3" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
     </row>
     <row r="235" spans="1:4">
@@ -40606,10 +40612,10 @@
         <v>2630</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>2807</v>
+        <v>2808</v>
       </c>
       <c r="C235" s="3" t="s">
-        <v>646</v>
+        <v>637</v>
       </c>
     </row>
     <row r="236" spans="1:4">
@@ -40617,10 +40623,10 @@
         <v>2630</v>
       </c>
       <c r="B236" s="3" t="s">
-        <v>2808</v>
+        <v>2809</v>
       </c>
       <c r="C236" s="3" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
     </row>
     <row r="237" spans="1:4">
@@ -40628,10 +40634,10 @@
         <v>2630</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>2809</v>
+        <v>2810</v>
       </c>
       <c r="C237" s="3" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
     </row>
     <row r="238" spans="1:4">
@@ -40639,10 +40645,10 @@
         <v>2630</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>2810</v>
+        <v>2811</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
     </row>
     <row r="239" spans="1:4">
@@ -40650,10 +40656,10 @@
         <v>2630</v>
       </c>
       <c r="B239" s="3" t="s">
-        <v>2811</v>
+        <v>2812</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>2812</v>
+        <v>657</v>
       </c>
     </row>
     <row r="240" spans="1:4">
@@ -40675,7 +40681,7 @@
         <v>2815</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>672</v>
+        <v>2816</v>
       </c>
     </row>
     <row r="242" spans="1:4">
@@ -40683,10 +40689,10 @@
         <v>2630</v>
       </c>
       <c r="B242" s="3" t="s">
-        <v>2816</v>
+        <v>2817</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>494</v>
+        <v>672</v>
       </c>
     </row>
     <row r="243" spans="1:4">
@@ -40694,10 +40700,10 @@
         <v>2630</v>
       </c>
       <c r="B243" s="3" t="s">
-        <v>2817</v>
+        <v>2818</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
     </row>
     <row r="244" spans="1:4">
@@ -40705,10 +40711,10 @@
         <v>2630</v>
       </c>
       <c r="B244" s="3" t="s">
-        <v>2818</v>
+        <v>2819</v>
       </c>
       <c r="C244" s="3" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
     </row>
     <row r="245" spans="1:4">
@@ -40716,10 +40722,10 @@
         <v>2630</v>
       </c>
       <c r="B245" s="3" t="s">
-        <v>2819</v>
+        <v>2820</v>
       </c>
       <c r="C245" s="3" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
     </row>
     <row r="246" spans="1:4">
@@ -40727,10 +40733,10 @@
         <v>2630</v>
       </c>
       <c r="B246" s="3" t="s">
-        <v>2820</v>
-      </c>
-      <c r="D246" s="3" t="s">
         <v>2821</v>
+      </c>
+      <c r="C246" s="3" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="247" spans="1:4">
@@ -40751,8 +40757,8 @@
       <c r="B248" s="3" t="s">
         <v>2824</v>
       </c>
-      <c r="C248" s="3" t="s">
-        <v>681</v>
+      <c r="D248" s="3" t="s">
+        <v>2825</v>
       </c>
     </row>
     <row r="249" spans="1:4">
@@ -40760,10 +40766,10 @@
         <v>2630</v>
       </c>
       <c r="B249" s="3" t="s">
-        <v>2825</v>
+        <v>2826</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>2826</v>
+        <v>681</v>
       </c>
     </row>
     <row r="250" spans="1:4">
@@ -40785,7 +40791,7 @@
         <v>2829</v>
       </c>
       <c r="C251" s="3" t="s">
-        <v>698</v>
+        <v>2830</v>
       </c>
     </row>
     <row r="252" spans="1:4">
@@ -40793,10 +40799,10 @@
         <v>2630</v>
       </c>
       <c r="B252" s="3" t="s">
-        <v>2830</v>
+        <v>2831</v>
       </c>
       <c r="C252" s="3" t="s">
-        <v>2831</v>
+        <v>698</v>
       </c>
     </row>
     <row r="253" spans="1:4">
@@ -40807,7 +40813,7 @@
         <v>2832</v>
       </c>
       <c r="C253" s="3" t="s">
-        <v>711</v>
+        <v>2833</v>
       </c>
     </row>
     <row r="254" spans="1:4">
@@ -40815,10 +40821,10 @@
         <v>2630</v>
       </c>
       <c r="B254" s="3" t="s">
-        <v>2833</v>
+        <v>2834</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>703</v>
+        <v>711</v>
       </c>
     </row>
     <row r="255" spans="1:4">
@@ -40826,10 +40832,10 @@
         <v>2630</v>
       </c>
       <c r="B255" s="3" t="s">
-        <v>2834</v>
+        <v>2835</v>
       </c>
       <c r="C255" s="3" t="s">
-        <v>719</v>
+        <v>703</v>
       </c>
     </row>
     <row r="256" spans="1:4">
@@ -40837,10 +40843,10 @@
         <v>2630</v>
       </c>
       <c r="B256" s="3" t="s">
-        <v>2835</v>
+        <v>2836</v>
       </c>
       <c r="C256" s="3" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
     </row>
     <row r="257" spans="1:4">
@@ -40848,10 +40854,10 @@
         <v>2630</v>
       </c>
       <c r="B257" s="3" t="s">
-        <v>2836</v>
+        <v>2837</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>2837</v>
+        <v>715</v>
       </c>
     </row>
     <row r="258" spans="1:4">
@@ -40862,7 +40868,7 @@
         <v>2838</v>
       </c>
       <c r="C258" s="3" t="s">
-        <v>728</v>
+        <v>2839</v>
       </c>
     </row>
     <row r="259" spans="1:4">
@@ -40870,10 +40876,10 @@
         <v>2630</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>2839</v>
+        <v>2840</v>
       </c>
       <c r="C259" s="3" t="s">
-        <v>759</v>
+        <v>728</v>
       </c>
     </row>
     <row r="260" spans="1:4">
@@ -40881,10 +40887,10 @@
         <v>2630</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>2840</v>
+        <v>2841</v>
       </c>
       <c r="C260" s="3" t="s">
-        <v>747</v>
+        <v>759</v>
       </c>
     </row>
     <row r="261" spans="1:4">
@@ -40892,10 +40898,10 @@
         <v>2630</v>
       </c>
       <c r="B261" s="3" t="s">
-        <v>2841</v>
+        <v>2842</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>768</v>
+        <v>747</v>
       </c>
     </row>
     <row r="262" spans="1:4">
@@ -40903,10 +40909,10 @@
         <v>2630</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>2842</v>
+        <v>2843</v>
       </c>
       <c r="C262" s="3" t="s">
-        <v>756</v>
+        <v>768</v>
       </c>
     </row>
     <row r="263" spans="1:4">
@@ -40914,10 +40920,10 @@
         <v>2630</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>2843</v>
+        <v>2844</v>
       </c>
       <c r="C263" s="3" t="s">
-        <v>737</v>
+        <v>756</v>
       </c>
     </row>
     <row r="264" spans="1:4">
@@ -40925,10 +40931,10 @@
         <v>2630</v>
       </c>
       <c r="B264" s="3" t="s">
-        <v>2844</v>
+        <v>2845</v>
       </c>
       <c r="C264" s="3" t="s">
-        <v>2845</v>
+        <v>737</v>
       </c>
     </row>
     <row r="265" spans="1:4">
@@ -40939,7 +40945,7 @@
         <v>2846</v>
       </c>
       <c r="C265" s="3" t="s">
-        <v>775</v>
+        <v>2847</v>
       </c>
     </row>
     <row r="266" spans="1:4">
@@ -40947,10 +40953,10 @@
         <v>2630</v>
       </c>
       <c r="B266" s="3" t="s">
-        <v>2847</v>
+        <v>2848</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>722</v>
+        <v>775</v>
       </c>
     </row>
     <row r="267" spans="1:4">
@@ -40958,10 +40964,10 @@
         <v>2630</v>
       </c>
       <c r="B267" s="3" t="s">
-        <v>2848</v>
+        <v>2849</v>
       </c>
       <c r="C267" s="3" t="s">
-        <v>733</v>
+        <v>722</v>
       </c>
     </row>
     <row r="268" spans="1:4">
@@ -40969,7 +40975,7 @@
         <v>2630</v>
       </c>
       <c r="B268" s="3" t="s">
-        <v>2849</v>
+        <v>2850</v>
       </c>
       <c r="C268" s="3" t="s">
         <v>733</v>
@@ -40980,21 +40986,21 @@
         <v>2630</v>
       </c>
       <c r="B269" s="3" t="s">
-        <v>2850</v>
+        <v>2851</v>
       </c>
       <c r="C269" s="3" t="s">
-        <v>781</v>
+        <v>733</v>
       </c>
     </row>
     <row r="270" spans="1:4">
       <c r="A270" s="3" t="s">
-        <v>615</v>
+        <v>2630</v>
       </c>
       <c r="B270" s="3" t="s">
-        <v>2851</v>
-      </c>
-      <c r="D270" s="3" t="s">
         <v>2852</v>
+      </c>
+      <c r="C270" s="3" t="s">
+        <v>781</v>
       </c>
     </row>
     <row r="271" spans="1:4">
@@ -41027,7 +41033,7 @@
         <v>2857</v>
       </c>
       <c r="D273" s="3" t="s">
-        <v>2852</v>
+        <v>2858</v>
       </c>
     </row>
     <row r="274" spans="1:4">
@@ -41035,10 +41041,10 @@
         <v>615</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>2858</v>
+        <v>2859</v>
       </c>
       <c r="D274" s="3" t="s">
-        <v>2852</v>
+        <v>2854</v>
       </c>
     </row>
     <row r="275" spans="1:4">
@@ -41046,10 +41052,10 @@
         <v>615</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>2859</v>
+        <v>2860</v>
       </c>
       <c r="D275" s="3" t="s">
-        <v>2852</v>
+        <v>2854</v>
       </c>
     </row>
     <row r="276" spans="1:4">
@@ -41057,10 +41063,10 @@
         <v>615</v>
       </c>
       <c r="B276" s="3" t="s">
-        <v>2860</v>
-      </c>
-      <c r="C276" s="3" t="s">
-        <v>490</v>
+        <v>2861</v>
+      </c>
+      <c r="D276" s="3" t="s">
+        <v>2854</v>
       </c>
     </row>
     <row r="277" spans="1:4">
@@ -41068,10 +41074,10 @@
         <v>615</v>
       </c>
       <c r="B277" s="3" t="s">
-        <v>2861</v>
-      </c>
-      <c r="D277" s="3" t="s">
         <v>2862</v>
+      </c>
+      <c r="C277" s="3" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -41181,11 +41187,22 @@
         <v>2881</v>
       </c>
       <c r="D287" s="3" t="s">
-        <v>2852</v>
+        <v>2882</v>
+      </c>
+    </row>
+    <row r="288" spans="1:4">
+      <c r="A288" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="B288" s="3" t="s">
+        <v>2883</v>
+      </c>
+      <c r="D288" s="3" t="s">
+        <v>2854</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D287"/>
+  <autoFilter ref="A1:D288"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not in the list" error="Pick one of: operation, job, schedule, handler." promptTitle="Kind" prompt="operation, job, schedule or handler" sqref="A2:A2001">
       <formula1>"operation,job,schedule,handler"</formula1>
@@ -41210,282 +41227,282 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>2882</v>
+        <v>2884</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2883</v>
+        <v>2885</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2884</v>
+        <v>2886</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>2885</v>
+        <v>2887</v>
       </c>
       <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2886</v>
+        <v>2888</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2887</v>
+        <v>2889</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>2888</v>
+        <v>2890</v>
       </c>
       <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2889</v>
+        <v>2891</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2890</v>
+        <v>2892</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>2888</v>
+        <v>2890</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2891</v>
+        <v>2893</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2892</v>
+        <v>2894</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>2888</v>
+        <v>2890</v>
       </c>
       <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2893</v>
+        <v>2895</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2894</v>
+        <v>2896</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2896</v>
+        <v>2898</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2897</v>
+        <v>2899</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2898</v>
+        <v>2900</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2899</v>
+        <v>2901</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>2900</v>
+        <v>2902</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2901</v>
+        <v>2903</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2902</v>
+        <v>2904</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2903</v>
+        <v>2905</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>2904</v>
+        <v>2906</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>2905</v>
+        <v>2907</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>2906</v>
+        <v>2908</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2907</v>
+        <v>2909</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>2908</v>
+        <v>2910</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>2909</v>
+        <v>2911</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>2910</v>
+        <v>2912</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>2911</v>
+        <v>2913</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2912</v>
+        <v>2914</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2913</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="3" t="s">
-        <v>2895</v>
+        <v>2897</v>
       </c>
       <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2914</v>
+        <v>2916</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="3" t="s">
-        <v>2916</v>
+        <v>2918</v>
       </c>
       <c r="B16" s="3">
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>2917</v>
+        <v>2919</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>2918</v>
+        <v>2920</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="3" t="s">
-        <v>2916</v>
+        <v>2918</v>
       </c>
       <c r="B17" s="3">
         <v>17</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2919</v>
+        <v>2921</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2920</v>
+        <v>2922</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="3" t="s">
-        <v>2916</v>
+        <v>2918</v>
       </c>
       <c r="B18" s="3">
         <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>2921</v>
+        <v>2923</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2922</v>
+        <v>2924</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="3" t="s">
-        <v>2923</v>
+        <v>2925</v>
       </c>
       <c r="B19" s="3">
         <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>2924</v>
+        <v>2926</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>2925</v>
+        <v>2927</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="3" t="s">
-        <v>2926</v>
+        <v>2928</v>
       </c>
       <c r="B20" s="3">
         <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>2927</v>
+        <v>2929</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>2928</v>
+        <v>2930</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(tracking,pages,assistant): patch 0021 is plan version 21; nested-emphasis step bound; readers line without names (#690 review)
Patch 0021 said plan_version 20, the same as #697's 0020, so applying it
replaced #697's changelog row. It is now 21 (added_in 21), regenerated from
next's plan: the diff against next only adds. The backtick scan counts its
steps, and the step test adds failing openers at every level of nesting,
bounded by ten looks per level. The readers line counts readers who are no
longer members instead of leaving their names blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Actors!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$291</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Enums!$A$1:$C$473</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Events!$A$1:$L$173</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8938" uniqueCount="2944">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8941" uniqueCount="2946">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -38,7 +38,7 @@
     <t>Plan version</t>
   </si>
   <si>
-    <t>20 (2026-10-28)</t>
+    <t>21 (2026-10-28)</t>
   </si>
   <si>
     <t>What this is</t>
@@ -8856,6 +8856,12 @@
   </si>
   <si>
     <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>You replied. Done? (campbooks-cloud#396): tasks.task_reply_noticed (a reply of the member in the conversation an open Do task came from) and tasks.task_reply_answered (the member answered Not yet); Coverage for tasks.notice_replies, tasks.answer_reply and tasks.unanswer_reply.</t>
+  </si>
+  <si>
+    <t>#697</t>
   </si>
   <si>
     <t>Mail and Scout in pages (campbooks-cloud#364): 2 pages events for files saved from a message (how many) and a section appended (how many blocks and sources, in buckets); 2 assistant tools (find_pages, read_page) and 2 proposal actions (append_section, new_page); Coverage for every operation of the change.</t>
@@ -13482,7 +13488,7 @@
         <v>522</v>
       </c>
       <c r="K106" s="3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L106" s="3" t="s">
         <v>523</v>
@@ -14242,7 +14248,7 @@
         <v>605</v>
       </c>
       <c r="K126" s="3">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="L126" s="3" t="s">
         <v>523</v>
@@ -41423,7 +41429,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12.7109375" customWidth="1"/>
@@ -41711,8 +41717,22 @@
         <v>2943</v>
       </c>
     </row>
+    <row r="21" spans="1:4">
+      <c r="A21" s="3" t="s">
+        <v>2941</v>
+      </c>
+      <c r="B21" s="3">
+        <v>21</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>2944</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>2945</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D20"/>
+  <autoFilter ref="A1:D21"/>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="YYYY-MM-DD" sqref="A2:A2001"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Plan version" prompt="From 1, one per change." sqref="B2:B2001"/>

</xml_diff>

<commit_message>
chore(tracking): Coverage for schedule.apply_calendar_list (patch 0027, cloud#405)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/tracking-plan.xlsx
+++ b/tracking/tracking-plan.xlsx
@@ -18,8 +18,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Actors!$A$1:$C$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$294</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">Changelog!$A$1:$D$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">Coverage!$A$1:$D$295</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Enums!$A$1:$C$477</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Events!$A$1:$L$174</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Properties!$A$1:$K$367</definedName>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8997" uniqueCount="2968">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9003" uniqueCount="2972">
   <si>
     <t>Campbooks tracking plan</t>
   </si>
@@ -38,7 +38,7 @@
     <t>Plan version</t>
   </si>
   <si>
-    <t>26 (2026-10-28)</t>
+    <t>27 (2026-10-31)</t>
   </si>
   <si>
     <t>What this is</t>
@@ -7721,6 +7721,9 @@
     <t>schedule.apply_calendar_changes</t>
   </si>
   <si>
+    <t>schedule.apply_calendar_list</t>
+  </si>
+  <si>
     <t>schedule.apply_outcome</t>
   </si>
   <si>
@@ -8934,6 +8937,15 @@
   </si>
   <si>
     <t>#705</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
+  </si>
+  <si>
+    <t>Calendars shared after connecting (campbooks-cloud#405): Coverage for schedule.apply_calendar_list, which tracks the calendars it adds as schedule.calendar_added.</t>
+  </si>
+  <si>
+    <t>#713</t>
   </si>
 </sst>
 </file>
@@ -38406,7 +38418,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D294"/>
+  <dimension ref="A1:D295"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -38921,7 +38933,7 @@
         <v>2563</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>149</v>
+        <v>614</v>
       </c>
     </row>
     <row r="47" spans="1:4">
@@ -38932,7 +38944,7 @@
         <v>2564</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>665</v>
+        <v>149</v>
       </c>
     </row>
     <row r="48" spans="1:4">
@@ -38942,8 +38954,8 @@
       <c r="B48" s="3" t="s">
         <v>2565</v>
       </c>
-      <c r="D48" s="3" t="s">
-        <v>2566</v>
+      <c r="C48" s="3" t="s">
+        <v>665</v>
       </c>
     </row>
     <row r="49" spans="1:4">
@@ -38951,10 +38963,10 @@
         <v>2490</v>
       </c>
       <c r="B49" s="3" t="s">
+        <v>2566</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>2567</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>614</v>
       </c>
     </row>
     <row r="50" spans="1:4">
@@ -38964,8 +38976,8 @@
       <c r="B50" s="3" t="s">
         <v>2568</v>
       </c>
-      <c r="D50" s="3" t="s">
-        <v>2494</v>
+      <c r="C50" s="3" t="s">
+        <v>614</v>
       </c>
     </row>
     <row r="51" spans="1:4">
@@ -38976,7 +38988,7 @@
         <v>2569</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>2570</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="52" spans="1:4">
@@ -38984,10 +38996,10 @@
         <v>2490</v>
       </c>
       <c r="B52" s="3" t="s">
+        <v>2570</v>
+      </c>
+      <c r="D52" s="3" t="s">
         <v>2571</v>
-      </c>
-      <c r="D52" s="3" t="s">
-        <v>2572</v>
       </c>
     </row>
     <row r="53" spans="1:4">
@@ -38995,10 +39007,10 @@
         <v>2490</v>
       </c>
       <c r="B53" s="3" t="s">
+        <v>2572</v>
+      </c>
+      <c r="D53" s="3" t="s">
         <v>2573</v>
-      </c>
-      <c r="D53" s="3" t="s">
-        <v>2574</v>
       </c>
     </row>
     <row r="54" spans="1:4">
@@ -39006,10 +39018,10 @@
         <v>2490</v>
       </c>
       <c r="B54" s="3" t="s">
+        <v>2574</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>2575</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>2576</v>
       </c>
     </row>
     <row r="55" spans="1:4">
@@ -39017,10 +39029,10 @@
         <v>2490</v>
       </c>
       <c r="B55" s="3" t="s">
+        <v>2576</v>
+      </c>
+      <c r="D55" s="3" t="s">
         <v>2577</v>
-      </c>
-      <c r="D55" s="3" t="s">
-        <v>2578</v>
       </c>
     </row>
     <row r="56" spans="1:4">
@@ -39028,10 +39040,10 @@
         <v>2490</v>
       </c>
       <c r="B56" s="3" t="s">
+        <v>2578</v>
+      </c>
+      <c r="D56" s="3" t="s">
         <v>2579</v>
-      </c>
-      <c r="D56" s="3" t="s">
-        <v>2580</v>
       </c>
     </row>
     <row r="57" spans="1:4">
@@ -39039,10 +39051,10 @@
         <v>2490</v>
       </c>
       <c r="B57" s="3" t="s">
+        <v>2580</v>
+      </c>
+      <c r="D57" s="3" t="s">
         <v>2581</v>
-      </c>
-      <c r="C57" s="3" t="s">
-        <v>2582</v>
       </c>
     </row>
     <row r="58" spans="1:4">
@@ -39050,10 +39062,10 @@
         <v>2490</v>
       </c>
       <c r="B58" s="3" t="s">
+        <v>2582</v>
+      </c>
+      <c r="C58" s="3" t="s">
         <v>2583</v>
-      </c>
-      <c r="C58" s="3" t="s">
-        <v>708</v>
       </c>
     </row>
     <row r="59" spans="1:4">
@@ -39064,7 +39076,7 @@
         <v>2584</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>2585</v>
+        <v>708</v>
       </c>
     </row>
     <row r="60" spans="1:4">
@@ -39072,10 +39084,10 @@
         <v>2490</v>
       </c>
       <c r="B60" s="3" t="s">
+        <v>2585</v>
+      </c>
+      <c r="C60" s="3" t="s">
         <v>2586</v>
-      </c>
-      <c r="C60" s="3" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="61" spans="1:4">
@@ -39086,7 +39098,7 @@
         <v>2587</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>732</v>
+        <v>703</v>
       </c>
     </row>
     <row r="62" spans="1:4">
@@ -39096,8 +39108,8 @@
       <c r="B62" s="3" t="s">
         <v>2588</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>2494</v>
+      <c r="C62" s="3" t="s">
+        <v>732</v>
       </c>
     </row>
     <row r="63" spans="1:4">
@@ -39107,8 +39119,8 @@
       <c r="B63" s="3" t="s">
         <v>2589</v>
       </c>
-      <c r="C63" s="3" t="s">
-        <v>754</v>
+      <c r="D63" s="3" t="s">
+        <v>2494</v>
       </c>
     </row>
     <row r="64" spans="1:4">
@@ -39119,18 +39131,18 @@
         <v>2590</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="3" t="s">
-        <v>496</v>
+        <v>2490</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>2591</v>
       </c>
-      <c r="D65" s="3" t="s">
-        <v>2592</v>
+      <c r="C65" s="3" t="s">
+        <v>757</v>
       </c>
     </row>
     <row r="66" spans="1:4">
@@ -39138,10 +39150,10 @@
         <v>496</v>
       </c>
       <c r="B66" s="3" t="s">
+        <v>2592</v>
+      </c>
+      <c r="D66" s="3" t="s">
         <v>2593</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>2594</v>
       </c>
     </row>
     <row r="67" spans="1:4">
@@ -39149,10 +39161,10 @@
         <v>496</v>
       </c>
       <c r="B67" s="3" t="s">
+        <v>2594</v>
+      </c>
+      <c r="D67" s="3" t="s">
         <v>2595</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>2596</v>
       </c>
     </row>
     <row r="68" spans="1:4">
@@ -39160,10 +39172,10 @@
         <v>496</v>
       </c>
       <c r="B68" s="3" t="s">
+        <v>2596</v>
+      </c>
+      <c r="D68" s="3" t="s">
         <v>2597</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>2598</v>
       </c>
     </row>
     <row r="69" spans="1:4">
@@ -39171,10 +39183,10 @@
         <v>496</v>
       </c>
       <c r="B69" s="3" t="s">
+        <v>2598</v>
+      </c>
+      <c r="D69" s="3" t="s">
         <v>2599</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:4">
@@ -39185,7 +39197,7 @@
         <v>2600</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>2601</v>
+        <v>144</v>
       </c>
     </row>
     <row r="71" spans="1:4">
@@ -39193,10 +39205,10 @@
         <v>496</v>
       </c>
       <c r="B71" s="3" t="s">
+        <v>2601</v>
+      </c>
+      <c r="C71" s="3" t="s">
         <v>2602</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>2603</v>
       </c>
     </row>
     <row r="72" spans="1:4">
@@ -39204,10 +39216,10 @@
         <v>496</v>
       </c>
       <c r="B72" s="3" t="s">
+        <v>2603</v>
+      </c>
+      <c r="C72" s="3" t="s">
         <v>2604</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="73" spans="1:4">
@@ -39218,7 +39230,7 @@
         <v>2605</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>359</v>
+        <v>295</v>
       </c>
     </row>
     <row r="74" spans="1:4">
@@ -39228,8 +39240,8 @@
       <c r="B74" s="3" t="s">
         <v>2606</v>
       </c>
-      <c r="D74" s="3" t="s">
-        <v>2607</v>
+      <c r="C74" s="3" t="s">
+        <v>359</v>
       </c>
     </row>
     <row r="75" spans="1:4">
@@ -39237,10 +39249,10 @@
         <v>496</v>
       </c>
       <c r="B75" s="3" t="s">
+        <v>2607</v>
+      </c>
+      <c r="D75" s="3" t="s">
         <v>2608</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="76" spans="1:4">
@@ -39251,7 +39263,7 @@
         <v>2609</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>300</v>
+        <v>271</v>
       </c>
     </row>
     <row r="77" spans="1:4">
@@ -39261,8 +39273,8 @@
       <c r="B77" s="3" t="s">
         <v>2610</v>
       </c>
-      <c r="D77" s="3" t="s">
-        <v>2611</v>
+      <c r="C77" s="3" t="s">
+        <v>300</v>
       </c>
     </row>
     <row r="78" spans="1:4">
@@ -39270,10 +39282,10 @@
         <v>496</v>
       </c>
       <c r="B78" s="3" t="s">
+        <v>2611</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>2612</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>2613</v>
       </c>
     </row>
     <row r="79" spans="1:4">
@@ -39281,10 +39293,10 @@
         <v>496</v>
       </c>
       <c r="B79" s="3" t="s">
+        <v>2613</v>
+      </c>
+      <c r="D79" s="3" t="s">
         <v>2614</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>2615</v>
       </c>
     </row>
     <row r="80" spans="1:4">
@@ -39292,10 +39304,10 @@
         <v>496</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>2615</v>
+      </c>
+      <c r="D80" s="3" t="s">
         <v>2616</v>
-      </c>
-      <c r="C80" s="3" t="s">
-        <v>305</v>
       </c>
     </row>
     <row r="81" spans="1:4">
@@ -39316,8 +39328,8 @@
       <c r="B82" s="3" t="s">
         <v>2618</v>
       </c>
-      <c r="D82" s="3" t="s">
-        <v>2607</v>
+      <c r="C82" s="3" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="83" spans="1:4">
@@ -39327,8 +39339,8 @@
       <c r="B83" s="3" t="s">
         <v>2619</v>
       </c>
-      <c r="C83" s="3" t="s">
-        <v>2620</v>
+      <c r="D83" s="3" t="s">
+        <v>2608</v>
       </c>
     </row>
     <row r="84" spans="1:4">
@@ -39336,10 +39348,10 @@
         <v>496</v>
       </c>
       <c r="B84" s="3" t="s">
+        <v>2620</v>
+      </c>
+      <c r="C84" s="3" t="s">
         <v>2621</v>
-      </c>
-      <c r="D84" s="3" t="s">
-        <v>2622</v>
       </c>
     </row>
     <row r="85" spans="1:4">
@@ -39347,10 +39359,10 @@
         <v>496</v>
       </c>
       <c r="B85" s="3" t="s">
+        <v>2622</v>
+      </c>
+      <c r="D85" s="3" t="s">
         <v>2623</v>
-      </c>
-      <c r="D85" s="3" t="s">
-        <v>2624</v>
       </c>
     </row>
     <row r="86" spans="1:4">
@@ -39358,10 +39370,10 @@
         <v>496</v>
       </c>
       <c r="B86" s="3" t="s">
+        <v>2624</v>
+      </c>
+      <c r="D86" s="3" t="s">
         <v>2625</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="87" spans="1:4">
@@ -39371,8 +39383,8 @@
       <c r="B87" s="3" t="s">
         <v>2626</v>
       </c>
-      <c r="D87" s="3" t="s">
-        <v>2607</v>
+      <c r="C87" s="3" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="88" spans="1:4">
@@ -39383,7 +39395,7 @@
         <v>2627</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>2628</v>
+        <v>2608</v>
       </c>
     </row>
     <row r="89" spans="1:4">
@@ -39391,10 +39403,10 @@
         <v>496</v>
       </c>
       <c r="B89" s="3" t="s">
+        <v>2628</v>
+      </c>
+      <c r="D89" s="3" t="s">
         <v>2629</v>
-      </c>
-      <c r="D89" s="3" t="s">
-        <v>2630</v>
       </c>
     </row>
     <row r="90" spans="1:4">
@@ -39402,10 +39414,10 @@
         <v>496</v>
       </c>
       <c r="B90" s="3" t="s">
+        <v>2630</v>
+      </c>
+      <c r="D90" s="3" t="s">
         <v>2631</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>2632</v>
       </c>
     </row>
     <row r="91" spans="1:4">
@@ -39413,10 +39425,10 @@
         <v>496</v>
       </c>
       <c r="B91" s="3" t="s">
+        <v>2632</v>
+      </c>
+      <c r="D91" s="3" t="s">
         <v>2633</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>2634</v>
       </c>
     </row>
     <row r="92" spans="1:4">
@@ -39424,10 +39436,10 @@
         <v>496</v>
       </c>
       <c r="B92" s="3" t="s">
+        <v>2634</v>
+      </c>
+      <c r="D92" s="3" t="s">
         <v>2635</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>2636</v>
       </c>
     </row>
     <row r="93" spans="1:4">
@@ -39435,10 +39447,10 @@
         <v>496</v>
       </c>
       <c r="B93" s="3" t="s">
+        <v>2636</v>
+      </c>
+      <c r="D93" s="3" t="s">
         <v>2637</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>2638</v>
       </c>
     </row>
     <row r="94" spans="1:4">
@@ -39446,10 +39458,10 @@
         <v>496</v>
       </c>
       <c r="B94" s="3" t="s">
+        <v>2638</v>
+      </c>
+      <c r="D94" s="3" t="s">
         <v>2639</v>
-      </c>
-      <c r="D94" s="3" t="s">
-        <v>2640</v>
       </c>
     </row>
     <row r="95" spans="1:4">
@@ -39457,10 +39469,10 @@
         <v>496</v>
       </c>
       <c r="B95" s="3" t="s">
+        <v>2640</v>
+      </c>
+      <c r="D95" s="3" t="s">
         <v>2641</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>2642</v>
       </c>
     </row>
     <row r="96" spans="1:4">
@@ -39468,10 +39480,10 @@
         <v>496</v>
       </c>
       <c r="B96" s="3" t="s">
+        <v>2642</v>
+      </c>
+      <c r="D96" s="3" t="s">
         <v>2643</v>
-      </c>
-      <c r="C96" s="3" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="97" spans="1:4">
@@ -39492,8 +39504,8 @@
       <c r="B98" s="3" t="s">
         <v>2645</v>
       </c>
-      <c r="D98" s="3" t="s">
-        <v>2646</v>
+      <c r="C98" s="3" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="99" spans="1:4">
@@ -39501,10 +39513,10 @@
         <v>496</v>
       </c>
       <c r="B99" s="3" t="s">
+        <v>2646</v>
+      </c>
+      <c r="D99" s="3" t="s">
         <v>2647</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>2648</v>
       </c>
     </row>
     <row r="100" spans="1:4">
@@ -39512,10 +39524,10 @@
         <v>496</v>
       </c>
       <c r="B100" s="3" t="s">
+        <v>2648</v>
+      </c>
+      <c r="D100" s="3" t="s">
         <v>2649</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>2650</v>
       </c>
     </row>
     <row r="101" spans="1:4">
@@ -39523,10 +39535,10 @@
         <v>496</v>
       </c>
       <c r="B101" s="3" t="s">
+        <v>2650</v>
+      </c>
+      <c r="D101" s="3" t="s">
         <v>2651</v>
-      </c>
-      <c r="D101" s="3" t="s">
-        <v>2652</v>
       </c>
     </row>
     <row r="102" spans="1:4">
@@ -39534,125 +39546,125 @@
         <v>496</v>
       </c>
       <c r="B102" s="3" t="s">
+        <v>2652</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>2653</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>791</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B103" s="3" t="s">
         <v>2654</v>
       </c>
-      <c r="B103" s="3" t="s">
-        <v>2655</v>
-      </c>
       <c r="C103" s="3" t="s">
-        <v>2656</v>
+        <v>791</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B104" s="3" t="s">
+        <v>2656</v>
+      </c>
+      <c r="C104" s="3" t="s">
         <v>2657</v>
-      </c>
-      <c r="D104" s="3" t="s">
-        <v>2658</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B105" s="3" t="s">
+        <v>2658</v>
+      </c>
+      <c r="D105" s="3" t="s">
         <v>2659</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>2660</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>2661</v>
+        <v>85</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B107" s="3" t="s">
+        <v>2661</v>
+      </c>
+      <c r="C107" s="3" t="s">
         <v>2662</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>2663</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>2656</v>
+        <v>89</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>2664</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>93</v>
+        <v>2657</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>2665</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>2666</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>2667</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>2668</v>
@@ -39663,7 +39675,7 @@
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>2669</v>
@@ -39674,7 +39686,7 @@
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>2670</v>
@@ -39685,7 +39697,7 @@
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>2671</v>
@@ -39696,7 +39708,7 @@
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>2672</v>
@@ -39707,7 +39719,7 @@
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>2673</v>
@@ -39718,7 +39730,7 @@
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>2674</v>
@@ -39729,7 +39741,7 @@
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>2675</v>
@@ -39740,7 +39752,7 @@
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>2676</v>
@@ -39751,51 +39763,51 @@
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>2677</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>2678</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>2679</v>
+        <v>132</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B124" s="3" t="s">
+        <v>2679</v>
+      </c>
+      <c r="C124" s="3" t="s">
         <v>2680</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>2681</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B125" s="3" t="s">
+        <v>2681</v>
+      </c>
+      <c r="D125" s="3" t="s">
         <v>2682</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>121</v>
       </c>
     </row>
     <row r="126" spans="1:4">
       <c r="A126" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>2683</v>
@@ -39806,590 +39818,590 @@
     </row>
     <row r="127" spans="1:4">
       <c r="A127" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>2684</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>2685</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>2686</v>
+        <v>137</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B129" s="3" t="s">
+        <v>2686</v>
+      </c>
+      <c r="C129" s="3" t="s">
         <v>2687</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="130" spans="1:4">
       <c r="A130" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>2688</v>
       </c>
-      <c r="D130" s="3" t="s">
-        <v>2689</v>
+      <c r="C130" s="3" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="131" spans="1:4">
       <c r="A131" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B131" s="3" t="s">
+        <v>2689</v>
+      </c>
+      <c r="D131" s="3" t="s">
         <v>2690</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>2691</v>
       </c>
     </row>
     <row r="132" spans="1:4">
       <c r="A132" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B132" s="3" t="s">
+        <v>2691</v>
+      </c>
+      <c r="D132" s="3" t="s">
         <v>2692</v>
-      </c>
-      <c r="C132" s="3" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="133" spans="1:4">
       <c r="A133" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>2693</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>204</v>
+        <v>173</v>
       </c>
     </row>
     <row r="134" spans="1:4">
       <c r="A134" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>2694</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>348</v>
+        <v>204</v>
       </c>
     </row>
     <row r="135" spans="1:4">
       <c r="A135" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>2695</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>196</v>
+        <v>348</v>
       </c>
     </row>
     <row r="136" spans="1:4">
       <c r="A136" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>2696</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>279</v>
+        <v>196</v>
       </c>
     </row>
     <row r="137" spans="1:4">
       <c r="A137" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>2697</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>343</v>
+        <v>279</v>
       </c>
     </row>
     <row r="138" spans="1:4">
       <c r="A138" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>2698</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>312</v>
+        <v>343</v>
       </c>
     </row>
     <row r="139" spans="1:4">
       <c r="A139" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>2699</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>2700</v>
+        <v>312</v>
       </c>
     </row>
     <row r="140" spans="1:4">
       <c r="A140" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B140" s="3" t="s">
+        <v>2700</v>
+      </c>
+      <c r="C140" s="3" t="s">
         <v>2701</v>
-      </c>
-      <c r="C140" s="3" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="141" spans="1:4">
       <c r="A141" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>2702</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>2703</v>
+        <v>253</v>
       </c>
     </row>
     <row r="142" spans="1:4">
       <c r="A142" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B142" s="3" t="s">
+        <v>2703</v>
+      </c>
+      <c r="C142" s="3" t="s">
         <v>2704</v>
-      </c>
-      <c r="C142" s="3" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="143" spans="1:4">
       <c r="A143" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>2705</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>259</v>
+        <v>340</v>
       </c>
     </row>
     <row r="144" spans="1:4">
       <c r="A144" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>2706</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>324</v>
+        <v>259</v>
       </c>
     </row>
     <row r="145" spans="1:4">
       <c r="A145" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>2707</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>363</v>
+        <v>324</v>
       </c>
     </row>
     <row r="146" spans="1:4">
       <c r="A146" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B146" s="3" t="s">
         <v>2708</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>213</v>
+        <v>363</v>
       </c>
     </row>
     <row r="147" spans="1:4">
       <c r="A147" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B147" s="3" t="s">
         <v>2709</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>237</v>
+        <v>213</v>
       </c>
     </row>
     <row r="148" spans="1:4">
       <c r="A148" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B148" s="3" t="s">
         <v>2710</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>209</v>
+        <v>237</v>
       </c>
     </row>
     <row r="149" spans="1:4">
       <c r="A149" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B149" s="3" t="s">
         <v>2711</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>241</v>
+        <v>209</v>
       </c>
     </row>
     <row r="150" spans="1:4">
       <c r="A150" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B150" s="3" t="s">
         <v>2712</v>
       </c>
-      <c r="D150" s="3" t="s">
-        <v>2713</v>
+      <c r="C150" s="3" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="151" spans="1:4">
       <c r="A151" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B151" s="3" t="s">
+        <v>2713</v>
+      </c>
+      <c r="D151" s="3" t="s">
         <v>2714</v>
-      </c>
-      <c r="C151" s="3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="152" spans="1:4">
       <c r="A152" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B152" s="3" t="s">
         <v>2715</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>352</v>
+        <v>233</v>
       </c>
     </row>
     <row r="153" spans="1:4">
       <c r="A153" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>2716</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>316</v>
+        <v>352</v>
       </c>
     </row>
     <row r="154" spans="1:4">
       <c r="A154" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>2717</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>217</v>
+        <v>316</v>
       </c>
     </row>
     <row r="155" spans="1:4">
       <c r="A155" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>2718</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>309</v>
+        <v>217</v>
       </c>
     </row>
     <row r="156" spans="1:4">
       <c r="A156" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>2719</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
     </row>
     <row r="157" spans="1:4">
       <c r="A157" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>2720</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>2721</v>
+        <v>320</v>
       </c>
     </row>
     <row r="158" spans="1:4">
       <c r="A158" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B158" s="3" t="s">
+        <v>2721</v>
+      </c>
+      <c r="C158" s="3" t="s">
         <v>2722</v>
-      </c>
-      <c r="C158" s="3" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="159" spans="1:4">
       <c r="A159" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>2723</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>329</v>
+        <v>267</v>
       </c>
     </row>
     <row r="160" spans="1:4">
       <c r="A160" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>2724</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>221</v>
+        <v>329</v>
       </c>
     </row>
     <row r="161" spans="1:4">
       <c r="A161" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>2725</v>
       </c>
-      <c r="D161" s="3" t="s">
-        <v>2726</v>
+      <c r="C161" s="3" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="162" spans="1:4">
       <c r="A162" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B162" s="3" t="s">
+        <v>2726</v>
+      </c>
+      <c r="D162" s="3" t="s">
         <v>2727</v>
-      </c>
-      <c r="D162" s="3" t="s">
-        <v>2726</v>
       </c>
     </row>
     <row r="163" spans="1:4">
       <c r="A163" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>2728</v>
       </c>
-      <c r="C163" s="3" t="s">
-        <v>225</v>
+      <c r="D163" s="3" t="s">
+        <v>2727</v>
       </c>
     </row>
     <row r="164" spans="1:4">
       <c r="A164" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>2729</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
     </row>
     <row r="165" spans="1:4">
       <c r="A165" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>2730</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
     </row>
     <row r="166" spans="1:4">
       <c r="A166" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>2731</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
     </row>
     <row r="167" spans="1:4">
       <c r="A167" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>2732</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>284</v>
+        <v>249</v>
       </c>
     </row>
     <row r="168" spans="1:4">
       <c r="A168" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>2733</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>2734</v>
+        <v>284</v>
       </c>
     </row>
     <row r="169" spans="1:4">
       <c r="A169" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B169" s="3" t="s">
+        <v>2734</v>
+      </c>
+      <c r="C169" s="3" t="s">
         <v>2735</v>
-      </c>
-      <c r="C169" s="3" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="170" spans="1:4">
       <c r="A170" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>2736</v>
       </c>
-      <c r="D170" s="3" t="s">
-        <v>2726</v>
+      <c r="C170" s="3" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="171" spans="1:4">
       <c r="A171" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>2737</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>2726</v>
+        <v>2727</v>
       </c>
     </row>
     <row r="172" spans="1:4">
       <c r="A172" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>2738</v>
       </c>
-      <c r="C172" s="3" t="s">
-        <v>377</v>
+      <c r="D172" s="3" t="s">
+        <v>2727</v>
       </c>
     </row>
     <row r="173" spans="1:4">
       <c r="A173" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>2739</v>
       </c>
       <c r="C173" s="3" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="174" spans="1:4">
       <c r="A174" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>2740</v>
       </c>
       <c r="C174" s="3" t="s">
-        <v>2741</v>
+        <v>381</v>
       </c>
     </row>
     <row r="175" spans="1:4">
       <c r="A175" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B175" s="3" t="s">
+        <v>2741</v>
+      </c>
+      <c r="C175" s="3" t="s">
         <v>2742</v>
-      </c>
-      <c r="C175" s="3" t="s">
-        <v>2743</v>
       </c>
     </row>
     <row r="176" spans="1:4">
       <c r="A176" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B176" s="3" t="s">
+        <v>2743</v>
+      </c>
+      <c r="C176" s="3" t="s">
         <v>2744</v>
       </c>
-      <c r="D176" s="3" t="s">
+    </row>
+    <row r="177" spans="1:4">
+      <c r="A177" s="3" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B177" s="3" t="s">
         <v>2745</v>
       </c>
-    </row>
-    <row r="177" spans="1:3">
-      <c r="A177" s="3" t="s">
-        <v>2654</v>
-      </c>
-      <c r="B177" s="3" t="s">
+      <c r="D177" s="3" t="s">
         <v>2746</v>
       </c>
-      <c r="C177" s="3" t="s">
+    </row>
+    <row r="178" spans="1:4">
+      <c r="A178" s="3" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B178" s="3" t="s">
         <v>2747</v>
       </c>
-    </row>
-    <row r="178" spans="1:3">
-      <c r="A178" s="3" t="s">
-        <v>2654</v>
-      </c>
-      <c r="B178" s="3" t="s">
+      <c r="C178" s="3" t="s">
         <v>2748</v>
       </c>
-      <c r="C178" s="3" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3">
+    </row>
+    <row r="179" spans="1:4">
       <c r="A179" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>2749</v>
       </c>
       <c r="C179" s="3" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="180" spans="1:3">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4">
       <c r="A180" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>2750</v>
@@ -40398,504 +40410,504 @@
         <v>466</v>
       </c>
     </row>
-    <row r="181" spans="1:3">
+    <row r="181" spans="1:4">
       <c r="A181" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>2751</v>
       </c>
       <c r="C181" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="182" spans="1:4">
+      <c r="A182" s="3" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B182" s="3" t="s">
         <v>2752</v>
       </c>
-    </row>
-    <row r="182" spans="1:3">
-      <c r="A182" s="3" t="s">
-        <v>2654</v>
-      </c>
-      <c r="B182" s="3" t="s">
+      <c r="C182" s="3" t="s">
         <v>2753</v>
       </c>
-      <c r="C182" s="3" t="s">
+    </row>
+    <row r="183" spans="1:4">
+      <c r="A183" s="3" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B183" s="3" t="s">
         <v>2754</v>
       </c>
-    </row>
-    <row r="183" spans="1:3">
-      <c r="A183" s="3" t="s">
-        <v>2654</v>
-      </c>
-      <c r="B183" s="3" t="s">
+      <c r="C183" s="3" t="s">
         <v>2755</v>
       </c>
-      <c r="C183" s="3" t="s">
+    </row>
+    <row r="184" spans="1:4">
+      <c r="A184" s="3" t="s">
+        <v>2655</v>
+      </c>
+      <c r="B184" s="3" t="s">
         <v>2756</v>
       </c>
-    </row>
-    <row r="184" spans="1:3">
-      <c r="A184" s="3" t="s">
-        <v>2654</v>
-      </c>
-      <c r="B184" s="3" t="s">
+      <c r="C184" s="3" t="s">
         <v>2757</v>
       </c>
-      <c r="C184" s="3" t="s">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="185" spans="1:3">
+    </row>
+    <row r="185" spans="1:4">
       <c r="A185" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>2758</v>
       </c>
       <c r="C185" s="3" t="s">
-        <v>385</v>
-      </c>
-    </row>
-    <row r="186" spans="1:3">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4">
       <c r="A186" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>2759</v>
       </c>
       <c r="C186" s="3" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4">
       <c r="A187" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>2760</v>
       </c>
       <c r="C187" s="3" t="s">
-        <v>390</v>
-      </c>
-    </row>
-    <row r="188" spans="1:3">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4">
       <c r="A188" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>2761</v>
       </c>
       <c r="C188" s="3" t="s">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="189" spans="1:3">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4">
       <c r="A189" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>2762</v>
       </c>
       <c r="C189" s="3" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="190" spans="1:3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="190" spans="1:4">
       <c r="A190" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>2763</v>
       </c>
       <c r="C190" s="3" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4">
       <c r="A191" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>2764</v>
       </c>
       <c r="C191" s="3" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="192" spans="1:3">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4">
       <c r="A192" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>2765</v>
       </c>
       <c r="C192" s="3" t="s">
-        <v>410</v>
+        <v>462</v>
       </c>
     </row>
     <row r="193" spans="1:4">
       <c r="A193" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>2766</v>
       </c>
       <c r="C193" s="3" t="s">
-        <v>393</v>
+        <v>410</v>
       </c>
     </row>
     <row r="194" spans="1:4">
       <c r="A194" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>2767</v>
       </c>
       <c r="C194" s="3" t="s">
-        <v>470</v>
+        <v>393</v>
       </c>
     </row>
     <row r="195" spans="1:4">
       <c r="A195" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B195" s="3" t="s">
         <v>2768</v>
       </c>
-      <c r="D195" s="3" t="s">
-        <v>2769</v>
+      <c r="C195" s="3" t="s">
+        <v>470</v>
       </c>
     </row>
     <row r="196" spans="1:4">
       <c r="A196" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B196" s="3" t="s">
+        <v>2769</v>
+      </c>
+      <c r="D196" s="3" t="s">
         <v>2770</v>
-      </c>
-      <c r="D196" s="3" t="s">
-        <v>2771</v>
       </c>
     </row>
     <row r="197" spans="1:4">
       <c r="A197" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B197" s="3" t="s">
+        <v>2771</v>
+      </c>
+      <c r="D197" s="3" t="s">
         <v>2772</v>
-      </c>
-      <c r="D197" s="3" t="s">
-        <v>2773</v>
       </c>
     </row>
     <row r="198" spans="1:4">
       <c r="A198" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B198" s="3" t="s">
+        <v>2773</v>
+      </c>
+      <c r="D198" s="3" t="s">
         <v>2774</v>
-      </c>
-      <c r="D198" s="3" t="s">
-        <v>2775</v>
       </c>
     </row>
     <row r="199" spans="1:4">
       <c r="A199" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B199" s="3" t="s">
+        <v>2775</v>
+      </c>
+      <c r="D199" s="3" t="s">
         <v>2776</v>
-      </c>
-      <c r="D199" s="3" t="s">
-        <v>2777</v>
       </c>
     </row>
     <row r="200" spans="1:4">
       <c r="A200" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B200" s="3" t="s">
+        <v>2777</v>
+      </c>
+      <c r="D200" s="3" t="s">
         <v>2778</v>
-      </c>
-      <c r="C200" s="3" t="s">
-        <v>2779</v>
       </c>
     </row>
     <row r="201" spans="1:4">
       <c r="A201" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B201" s="3" t="s">
+        <v>2779</v>
+      </c>
+      <c r="C201" s="3" t="s">
         <v>2780</v>
-      </c>
-      <c r="C201" s="3" t="s">
-        <v>592</v>
       </c>
     </row>
     <row r="202" spans="1:4">
       <c r="A202" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B202" s="3" t="s">
         <v>2781</v>
       </c>
       <c r="C202" s="3" t="s">
-        <v>2782</v>
+        <v>592</v>
       </c>
     </row>
     <row r="203" spans="1:4">
       <c r="A203" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B203" s="3" t="s">
+        <v>2782</v>
+      </c>
+      <c r="C203" s="3" t="s">
         <v>2783</v>
-      </c>
-      <c r="C203" s="3" t="s">
-        <v>601</v>
       </c>
     </row>
     <row r="204" spans="1:4">
       <c r="A204" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B204" s="3" t="s">
         <v>2784</v>
       </c>
       <c r="C204" s="3" t="s">
-        <v>518</v>
+        <v>601</v>
       </c>
     </row>
     <row r="205" spans="1:4">
       <c r="A205" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B205" s="3" t="s">
         <v>2785</v>
       </c>
       <c r="C205" s="3" t="s">
-        <v>562</v>
+        <v>518</v>
       </c>
     </row>
     <row r="206" spans="1:4">
       <c r="A206" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B206" s="3" t="s">
         <v>2786</v>
       </c>
       <c r="C206" s="3" t="s">
-        <v>2787</v>
+        <v>562</v>
       </c>
     </row>
     <row r="207" spans="1:4">
       <c r="A207" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B207" s="3" t="s">
+        <v>2787</v>
+      </c>
+      <c r="C207" s="3" t="s">
         <v>2788</v>
-      </c>
-      <c r="C207" s="3" t="s">
-        <v>610</v>
       </c>
     </row>
     <row r="208" spans="1:4">
       <c r="A208" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B208" s="3" t="s">
         <v>2789</v>
       </c>
-      <c r="D208" s="3" t="s">
-        <v>2790</v>
+      <c r="C208" s="3" t="s">
+        <v>610</v>
       </c>
     </row>
     <row r="209" spans="1:4">
       <c r="A209" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B209" s="3" t="s">
+        <v>2790</v>
+      </c>
+      <c r="D209" s="3" t="s">
         <v>2791</v>
-      </c>
-      <c r="D209" s="3" t="s">
-        <v>2792</v>
       </c>
     </row>
     <row r="210" spans="1:4">
       <c r="A210" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B210" s="3" t="s">
+        <v>2792</v>
+      </c>
+      <c r="D210" s="3" t="s">
         <v>2793</v>
-      </c>
-      <c r="D210" s="3" t="s">
-        <v>2794</v>
       </c>
     </row>
     <row r="211" spans="1:4">
       <c r="A211" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B211" s="3" t="s">
+        <v>2794</v>
+      </c>
+      <c r="D211" s="3" t="s">
         <v>2795</v>
-      </c>
-      <c r="C211" s="3" t="s">
-        <v>2796</v>
       </c>
     </row>
     <row r="212" spans="1:4">
       <c r="A212" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B212" s="3" t="s">
+        <v>2796</v>
+      </c>
+      <c r="C212" s="3" t="s">
         <v>2797</v>
-      </c>
-      <c r="C212" s="3" t="s">
-        <v>571</v>
       </c>
     </row>
     <row r="213" spans="1:4">
       <c r="A213" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B213" s="3" t="s">
         <v>2798</v>
       </c>
       <c r="C213" s="3" t="s">
-        <v>574</v>
+        <v>571</v>
       </c>
     </row>
     <row r="214" spans="1:4">
       <c r="A214" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B214" s="3" t="s">
         <v>2799</v>
       </c>
       <c r="C214" s="3" t="s">
-        <v>596</v>
+        <v>574</v>
       </c>
     </row>
     <row r="215" spans="1:4">
       <c r="A215" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B215" s="3" t="s">
         <v>2800</v>
       </c>
-      <c r="D215" s="3" t="s">
-        <v>2801</v>
+      <c r="C215" s="3" t="s">
+        <v>596</v>
       </c>
     </row>
     <row r="216" spans="1:4">
       <c r="A216" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B216" s="3" t="s">
+        <v>2801</v>
+      </c>
+      <c r="D216" s="3" t="s">
         <v>2802</v>
-      </c>
-      <c r="D216" s="3" t="s">
-        <v>2803</v>
       </c>
     </row>
     <row r="217" spans="1:4">
       <c r="A217" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B217" s="3" t="s">
+        <v>2803</v>
+      </c>
+      <c r="D217" s="3" t="s">
         <v>2804</v>
-      </c>
-      <c r="D217" s="3" t="s">
-        <v>2805</v>
       </c>
     </row>
     <row r="218" spans="1:4">
       <c r="A218" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B218" s="3" t="s">
+        <v>2805</v>
+      </c>
+      <c r="D218" s="3" t="s">
         <v>2806</v>
-      </c>
-      <c r="C218" s="3" t="s">
-        <v>530</v>
       </c>
     </row>
     <row r="219" spans="1:4">
       <c r="A219" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B219" s="3" t="s">
         <v>2807</v>
       </c>
       <c r="C219" s="3" t="s">
-        <v>555</v>
+        <v>530</v>
       </c>
     </row>
     <row r="220" spans="1:4">
       <c r="A220" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B220" s="3" t="s">
         <v>2808</v>
       </c>
       <c r="C220" s="3" t="s">
-        <v>578</v>
+        <v>555</v>
       </c>
     </row>
     <row r="221" spans="1:4">
       <c r="A221" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B221" s="3" t="s">
         <v>2809</v>
       </c>
-      <c r="D221" s="3" t="s">
-        <v>2810</v>
+      <c r="C221" s="3" t="s">
+        <v>578</v>
       </c>
     </row>
     <row r="222" spans="1:4">
       <c r="A222" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B222" s="3" t="s">
+        <v>2810</v>
+      </c>
+      <c r="D222" s="3" t="s">
         <v>2811</v>
-      </c>
-      <c r="C222" s="3" t="s">
-        <v>511</v>
       </c>
     </row>
     <row r="223" spans="1:4">
       <c r="A223" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B223" s="3" t="s">
         <v>2812</v>
       </c>
-      <c r="D223" s="3" t="s">
-        <v>2813</v>
+      <c r="C223" s="3" t="s">
+        <v>511</v>
       </c>
     </row>
     <row r="224" spans="1:4">
       <c r="A224" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B224" s="3" t="s">
+        <v>2813</v>
+      </c>
+      <c r="D224" s="3" t="s">
         <v>2814</v>
-      </c>
-      <c r="C224" s="3" t="s">
-        <v>581</v>
       </c>
     </row>
     <row r="225" spans="1:4">
       <c r="A225" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B225" s="3" t="s">
         <v>2815</v>
       </c>
       <c r="C225" s="3" t="s">
-        <v>547</v>
+        <v>581</v>
       </c>
     </row>
     <row r="226" spans="1:4">
       <c r="A226" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B226" s="3" t="s">
         <v>2816</v>
@@ -40906,524 +40918,524 @@
     </row>
     <row r="227" spans="1:4">
       <c r="A227" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B227" s="3" t="s">
         <v>2817</v>
       </c>
-      <c r="D227" s="3" t="s">
-        <v>2818</v>
+      <c r="C227" s="3" t="s">
+        <v>547</v>
       </c>
     </row>
     <row r="228" spans="1:4">
       <c r="A228" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B228" s="3" t="s">
+        <v>2818</v>
+      </c>
+      <c r="D228" s="3" t="s">
         <v>2819</v>
-      </c>
-      <c r="C228" s="3" t="s">
-        <v>585</v>
       </c>
     </row>
     <row r="229" spans="1:4">
       <c r="A229" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B229" s="3" t="s">
         <v>2820</v>
       </c>
-      <c r="D229" s="3" t="s">
-        <v>2821</v>
+      <c r="C229" s="3" t="s">
+        <v>585</v>
       </c>
     </row>
     <row r="230" spans="1:4">
       <c r="A230" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B230" s="3" t="s">
+        <v>2821</v>
+      </c>
+      <c r="D230" s="3" t="s">
         <v>2822</v>
-      </c>
-      <c r="C230" s="3" t="s">
-        <v>524</v>
       </c>
     </row>
     <row r="231" spans="1:4">
       <c r="A231" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B231" s="3" t="s">
         <v>2823</v>
       </c>
       <c r="C231" s="3" t="s">
-        <v>551</v>
+        <v>524</v>
       </c>
     </row>
     <row r="232" spans="1:4">
       <c r="A232" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B232" s="3" t="s">
         <v>2824</v>
       </c>
       <c r="C232" s="3" t="s">
-        <v>588</v>
+        <v>551</v>
       </c>
     </row>
     <row r="233" spans="1:4">
       <c r="A233" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B233" s="3" t="s">
         <v>2825</v>
       </c>
       <c r="C233" s="3" t="s">
-        <v>568</v>
+        <v>588</v>
       </c>
     </row>
     <row r="234" spans="1:4">
       <c r="A234" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B234" s="3" t="s">
         <v>2826</v>
       </c>
-      <c r="D234" s="3" t="s">
-        <v>2827</v>
+      <c r="C234" s="3" t="s">
+        <v>568</v>
       </c>
     </row>
     <row r="235" spans="1:4">
       <c r="A235" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B235" s="3" t="s">
+        <v>2827</v>
+      </c>
+      <c r="D235" s="3" t="s">
         <v>2828</v>
-      </c>
-      <c r="D235" s="3" t="s">
-        <v>2829</v>
       </c>
     </row>
     <row r="236" spans="1:4">
       <c r="A236" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B236" s="3" t="s">
+        <v>2829</v>
+      </c>
+      <c r="D236" s="3" t="s">
         <v>2830</v>
-      </c>
-      <c r="D236" s="3" t="s">
-        <v>2831</v>
       </c>
     </row>
     <row r="237" spans="1:4">
       <c r="A237" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B237" s="3" t="s">
+        <v>2831</v>
+      </c>
+      <c r="D237" s="3" t="s">
         <v>2832</v>
-      </c>
-      <c r="C237" s="3" t="s">
-        <v>633</v>
       </c>
     </row>
     <row r="238" spans="1:4">
       <c r="A238" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B238" s="3" t="s">
         <v>2833</v>
       </c>
       <c r="C238" s="3" t="s">
-        <v>637</v>
+        <v>633</v>
       </c>
     </row>
     <row r="239" spans="1:4">
       <c r="A239" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B239" s="3" t="s">
         <v>2834</v>
       </c>
       <c r="C239" s="3" t="s">
-        <v>646</v>
+        <v>637</v>
       </c>
     </row>
     <row r="240" spans="1:4">
       <c r="A240" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B240" s="3" t="s">
         <v>2835</v>
       </c>
       <c r="C240" s="3" t="s">
-        <v>650</v>
+        <v>646</v>
       </c>
     </row>
     <row r="241" spans="1:4">
       <c r="A241" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B241" s="3" t="s">
         <v>2836</v>
       </c>
       <c r="C241" s="3" t="s">
-        <v>654</v>
+        <v>650</v>
       </c>
     </row>
     <row r="242" spans="1:4">
       <c r="A242" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B242" s="3" t="s">
         <v>2837</v>
       </c>
       <c r="C242" s="3" t="s">
-        <v>657</v>
+        <v>654</v>
       </c>
     </row>
     <row r="243" spans="1:4">
       <c r="A243" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B243" s="3" t="s">
         <v>2838</v>
       </c>
       <c r="C243" s="3" t="s">
-        <v>2839</v>
+        <v>657</v>
       </c>
     </row>
     <row r="244" spans="1:4">
       <c r="A244" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B244" s="3" t="s">
+        <v>2839</v>
+      </c>
+      <c r="C244" s="3" t="s">
         <v>2840</v>
-      </c>
-      <c r="C244" s="3" t="s">
-        <v>2841</v>
       </c>
     </row>
     <row r="245" spans="1:4">
       <c r="A245" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B245" s="3" t="s">
+        <v>2841</v>
+      </c>
+      <c r="C245" s="3" t="s">
         <v>2842</v>
-      </c>
-      <c r="C245" s="3" t="s">
-        <v>677</v>
       </c>
     </row>
     <row r="246" spans="1:4">
       <c r="A246" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B246" s="3" t="s">
         <v>2843</v>
       </c>
       <c r="C246" s="3" t="s">
-        <v>494</v>
+        <v>677</v>
       </c>
     </row>
     <row r="247" spans="1:4">
       <c r="A247" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B247" s="3" t="s">
         <v>2844</v>
       </c>
       <c r="C247" s="3" t="s">
-        <v>507</v>
+        <v>494</v>
       </c>
     </row>
     <row r="248" spans="1:4">
       <c r="A248" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B248" s="3" t="s">
         <v>2845</v>
       </c>
       <c r="C248" s="3" t="s">
-        <v>499</v>
+        <v>507</v>
       </c>
     </row>
     <row r="249" spans="1:4">
       <c r="A249" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B249" s="3" t="s">
         <v>2846</v>
       </c>
       <c r="C249" s="3" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
     </row>
     <row r="250" spans="1:4">
       <c r="A250" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B250" s="3" t="s">
         <v>2847</v>
       </c>
-      <c r="D250" s="3" t="s">
-        <v>2848</v>
+      <c r="C250" s="3" t="s">
+        <v>503</v>
       </c>
     </row>
     <row r="251" spans="1:4">
       <c r="A251" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B251" s="3" t="s">
+        <v>2848</v>
+      </c>
+      <c r="D251" s="3" t="s">
         <v>2849</v>
-      </c>
-      <c r="D251" s="3" t="s">
-        <v>2850</v>
       </c>
     </row>
     <row r="252" spans="1:4">
       <c r="A252" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B252" s="3" t="s">
+        <v>2850</v>
+      </c>
+      <c r="D252" s="3" t="s">
         <v>2851</v>
-      </c>
-      <c r="C252" s="3" t="s">
-        <v>727</v>
       </c>
     </row>
     <row r="253" spans="1:4">
       <c r="A253" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B253" s="3" t="s">
         <v>2852</v>
       </c>
       <c r="C253" s="3" t="s">
-        <v>686</v>
+        <v>727</v>
       </c>
     </row>
     <row r="254" spans="1:4">
       <c r="A254" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B254" s="3" t="s">
         <v>2853</v>
       </c>
       <c r="C254" s="3" t="s">
-        <v>2854</v>
+        <v>686</v>
       </c>
     </row>
     <row r="255" spans="1:4">
       <c r="A255" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B255" s="3" t="s">
+        <v>2854</v>
+      </c>
+      <c r="C255" s="3" t="s">
         <v>2855</v>
-      </c>
-      <c r="C255" s="3" t="s">
-        <v>2856</v>
       </c>
     </row>
     <row r="256" spans="1:4">
       <c r="A256" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B256" s="3" t="s">
+        <v>2856</v>
+      </c>
+      <c r="C256" s="3" t="s">
         <v>2857</v>
-      </c>
-      <c r="C256" s="3" t="s">
-        <v>703</v>
       </c>
     </row>
     <row r="257" spans="1:4">
       <c r="A257" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B257" s="3" t="s">
         <v>2858</v>
       </c>
       <c r="C257" s="3" t="s">
-        <v>2859</v>
+        <v>703</v>
       </c>
     </row>
     <row r="258" spans="1:4">
       <c r="A258" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B258" s="3" t="s">
+        <v>2859</v>
+      </c>
+      <c r="C258" s="3" t="s">
         <v>2860</v>
-      </c>
-      <c r="C258" s="3" t="s">
-        <v>716</v>
       </c>
     </row>
     <row r="259" spans="1:4">
       <c r="A259" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B259" s="3" t="s">
         <v>2861</v>
       </c>
       <c r="C259" s="3" t="s">
-        <v>708</v>
+        <v>716</v>
       </c>
     </row>
     <row r="260" spans="1:4">
       <c r="A260" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B260" s="3" t="s">
         <v>2862</v>
       </c>
       <c r="C260" s="3" t="s">
-        <v>724</v>
+        <v>708</v>
       </c>
     </row>
     <row r="261" spans="1:4">
       <c r="A261" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B261" s="3" t="s">
         <v>2863</v>
       </c>
       <c r="C261" s="3" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
     </row>
     <row r="262" spans="1:4">
       <c r="A262" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B262" s="3" t="s">
         <v>2864</v>
       </c>
-      <c r="D262" s="3" t="s">
-        <v>2865</v>
+      <c r="C262" s="3" t="s">
+        <v>720</v>
       </c>
     </row>
     <row r="263" spans="1:4">
       <c r="A263" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B263" s="3" t="s">
+        <v>2865</v>
+      </c>
+      <c r="D263" s="3" t="s">
         <v>2866</v>
-      </c>
-      <c r="C263" s="3" t="s">
-        <v>2867</v>
       </c>
     </row>
     <row r="264" spans="1:4">
       <c r="A264" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B264" s="3" t="s">
+        <v>2867</v>
+      </c>
+      <c r="C264" s="3" t="s">
         <v>2868</v>
-      </c>
-      <c r="C264" s="3" t="s">
-        <v>742</v>
       </c>
     </row>
     <row r="265" spans="1:4">
       <c r="A265" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B265" s="3" t="s">
         <v>2869</v>
       </c>
       <c r="C265" s="3" t="s">
-        <v>772</v>
+        <v>742</v>
       </c>
     </row>
     <row r="266" spans="1:4">
       <c r="A266" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B266" s="3" t="s">
         <v>2870</v>
       </c>
       <c r="C266" s="3" t="s">
-        <v>760</v>
+        <v>772</v>
       </c>
     </row>
     <row r="267" spans="1:4">
       <c r="A267" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B267" s="3" t="s">
         <v>2871</v>
       </c>
       <c r="C267" s="3" t="s">
-        <v>781</v>
+        <v>760</v>
       </c>
     </row>
     <row r="268" spans="1:4">
       <c r="A268" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B268" s="3" t="s">
         <v>2872</v>
       </c>
       <c r="C268" s="3" t="s">
-        <v>769</v>
+        <v>781</v>
       </c>
     </row>
     <row r="269" spans="1:4">
       <c r="A269" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B269" s="3" t="s">
         <v>2873</v>
       </c>
       <c r="C269" s="3" t="s">
-        <v>751</v>
+        <v>769</v>
       </c>
     </row>
     <row r="270" spans="1:4">
       <c r="A270" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B270" s="3" t="s">
         <v>2874</v>
       </c>
       <c r="C270" s="3" t="s">
-        <v>2875</v>
+        <v>751</v>
       </c>
     </row>
     <row r="271" spans="1:4">
       <c r="A271" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B271" s="3" t="s">
+        <v>2875</v>
+      </c>
+      <c r="C271" s="3" t="s">
         <v>2876</v>
-      </c>
-      <c r="C271" s="3" t="s">
-        <v>788</v>
       </c>
     </row>
     <row r="272" spans="1:4">
       <c r="A272" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B272" s="3" t="s">
         <v>2877</v>
       </c>
       <c r="C272" s="3" t="s">
-        <v>736</v>
+        <v>788</v>
       </c>
     </row>
     <row r="273" spans="1:4">
       <c r="A273" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B273" s="3" t="s">
         <v>2878</v>
       </c>
       <c r="C273" s="3" t="s">
-        <v>747</v>
+        <v>736</v>
       </c>
     </row>
     <row r="274" spans="1:4">
       <c r="A274" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B274" s="3" t="s">
         <v>2879</v>
@@ -41434,24 +41446,24 @@
     </row>
     <row r="275" spans="1:4">
       <c r="A275" s="3" t="s">
-        <v>2654</v>
+        <v>2655</v>
       </c>
       <c r="B275" s="3" t="s">
         <v>2880</v>
       </c>
       <c r="C275" s="3" t="s">
-        <v>794</v>
+        <v>747</v>
       </c>
     </row>
     <row r="276" spans="1:4">
       <c r="A276" s="3" t="s">
-        <v>615</v>
+        <v>2655</v>
       </c>
       <c r="B276" s="3" t="s">
         <v>2881</v>
       </c>
-      <c r="D276" s="3" t="s">
-        <v>2882</v>
+      <c r="C276" s="3" t="s">
+        <v>794</v>
       </c>
     </row>
     <row r="277" spans="1:4">
@@ -41459,10 +41471,10 @@
         <v>615</v>
       </c>
       <c r="B277" s="3" t="s">
+        <v>2882</v>
+      </c>
+      <c r="D277" s="3" t="s">
         <v>2883</v>
-      </c>
-      <c r="D277" s="3" t="s">
-        <v>2884</v>
       </c>
     </row>
     <row r="278" spans="1:4">
@@ -41470,10 +41482,10 @@
         <v>615</v>
       </c>
       <c r="B278" s="3" t="s">
+        <v>2884</v>
+      </c>
+      <c r="D278" s="3" t="s">
         <v>2885</v>
-      </c>
-      <c r="D278" s="3" t="s">
-        <v>2886</v>
       </c>
     </row>
     <row r="279" spans="1:4">
@@ -41481,10 +41493,10 @@
         <v>615</v>
       </c>
       <c r="B279" s="3" t="s">
+        <v>2886</v>
+      </c>
+      <c r="D279" s="3" t="s">
         <v>2887</v>
-      </c>
-      <c r="D279" s="3" t="s">
-        <v>2882</v>
       </c>
     </row>
     <row r="280" spans="1:4">
@@ -41495,7 +41507,7 @@
         <v>2888</v>
       </c>
       <c r="D280" s="3" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
     </row>
     <row r="281" spans="1:4">
@@ -41506,7 +41518,7 @@
         <v>2889</v>
       </c>
       <c r="D281" s="3" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
     </row>
     <row r="282" spans="1:4">
@@ -41517,7 +41529,7 @@
         <v>2890</v>
       </c>
       <c r="D282" s="3" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
     </row>
     <row r="283" spans="1:4">
@@ -41527,8 +41539,8 @@
       <c r="B283" s="3" t="s">
         <v>2891</v>
       </c>
-      <c r="C283" s="3" t="s">
-        <v>490</v>
+      <c r="D283" s="3" t="s">
+        <v>2883</v>
       </c>
     </row>
     <row r="284" spans="1:4">
@@ -41538,8 +41550,8 @@
       <c r="B284" s="3" t="s">
         <v>2892</v>
       </c>
-      <c r="D284" s="3" t="s">
-        <v>2893</v>
+      <c r="C284" s="3" t="s">
+        <v>490</v>
       </c>
     </row>
     <row r="285" spans="1:4">
@@ -41547,10 +41559,10 @@
         <v>615</v>
       </c>
       <c r="B285" s="3" t="s">
+        <v>2893</v>
+      </c>
+      <c r="D285" s="3" t="s">
         <v>2894</v>
-      </c>
-      <c r="D285" s="3" t="s">
-        <v>2895</v>
       </c>
     </row>
     <row r="286" spans="1:4">
@@ -41558,10 +41570,10 @@
         <v>615</v>
       </c>
       <c r="B286" s="3" t="s">
+        <v>2895</v>
+      </c>
+      <c r="D286" s="3" t="s">
         <v>2896</v>
-      </c>
-      <c r="D286" s="3" t="s">
-        <v>2897</v>
       </c>
     </row>
     <row r="287" spans="1:4">
@@ -41569,10 +41581,10 @@
         <v>615</v>
       </c>
       <c r="B287" s="3" t="s">
+        <v>2897</v>
+      </c>
+      <c r="D287" s="3" t="s">
         <v>2898</v>
-      </c>
-      <c r="D287" s="3" t="s">
-        <v>2899</v>
       </c>
     </row>
     <row r="288" spans="1:4">
@@ -41580,10 +41592,10 @@
         <v>615</v>
       </c>
       <c r="B288" s="3" t="s">
+        <v>2899</v>
+      </c>
+      <c r="D288" s="3" t="s">
         <v>2900</v>
-      </c>
-      <c r="D288" s="3" t="s">
-        <v>2901</v>
       </c>
     </row>
     <row r="289" spans="1:4">
@@ -41591,10 +41603,10 @@
         <v>615</v>
       </c>
       <c r="B289" s="3" t="s">
+        <v>2901</v>
+      </c>
+      <c r="D289" s="3" t="s">
         <v>2902</v>
-      </c>
-      <c r="D289" s="3" t="s">
-        <v>2903</v>
       </c>
     </row>
     <row r="290" spans="1:4">
@@ -41602,10 +41614,10 @@
         <v>615</v>
       </c>
       <c r="B290" s="3" t="s">
+        <v>2903</v>
+      </c>
+      <c r="D290" s="3" t="s">
         <v>2904</v>
-      </c>
-      <c r="D290" s="3" t="s">
-        <v>2905</v>
       </c>
     </row>
     <row r="291" spans="1:4">
@@ -41613,10 +41625,10 @@
         <v>615</v>
       </c>
       <c r="B291" s="3" t="s">
+        <v>2905</v>
+      </c>
+      <c r="D291" s="3" t="s">
         <v>2906</v>
-      </c>
-      <c r="D291" s="3" t="s">
-        <v>2907</v>
       </c>
     </row>
     <row r="292" spans="1:4">
@@ -41624,10 +41636,10 @@
         <v>615</v>
       </c>
       <c r="B292" s="3" t="s">
+        <v>2907</v>
+      </c>
+      <c r="D292" s="3" t="s">
         <v>2908</v>
-      </c>
-      <c r="D292" s="3" t="s">
-        <v>2909</v>
       </c>
     </row>
     <row r="293" spans="1:4">
@@ -41635,10 +41647,10 @@
         <v>615</v>
       </c>
       <c r="B293" s="3" t="s">
+        <v>2909</v>
+      </c>
+      <c r="D293" s="3" t="s">
         <v>2910</v>
-      </c>
-      <c r="D293" s="3" t="s">
-        <v>2911</v>
       </c>
     </row>
     <row r="294" spans="1:4">
@@ -41646,14 +41658,25 @@
         <v>615</v>
       </c>
       <c r="B294" s="3" t="s">
+        <v>2911</v>
+      </c>
+      <c r="D294" s="3" t="s">
         <v>2912</v>
       </c>
-      <c r="D294" s="3" t="s">
-        <v>2882</v>
+    </row>
+    <row r="295" spans="1:4">
+      <c r="A295" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="B295" s="3" t="s">
+        <v>2913</v>
+      </c>
+      <c r="D295" s="3" t="s">
+        <v>2883</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D294"/>
+  <autoFilter ref="A1:D295"/>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Not in the list" error="Pick one of: operation, job, schedule, handler." promptTitle="Kind" prompt="operation, job, schedule or handler" sqref="A2:A2001">
       <formula1>"operation,job,schedule,handler"</formula1>
@@ -41668,7 +41691,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="2" width="12.7109375" customWidth="1"/>
@@ -41678,342 +41701,356 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="4" t="s">
-        <v>2913</v>
+        <v>2914</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2914</v>
+        <v>2915</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>2915</v>
+        <v>2916</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="3" t="s">
-        <v>2916</v>
+        <v>2917</v>
       </c>
       <c r="B2" s="3">
         <v>1</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>2917</v>
+        <v>2918</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>2918</v>
+        <v>2919</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>2919</v>
+        <v>2920</v>
       </c>
       <c r="B3" s="3">
         <v>2</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>2920</v>
+        <v>2921</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>2921</v>
+        <v>2922</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>2919</v>
+        <v>2920</v>
       </c>
       <c r="B4" s="3">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>2922</v>
+        <v>2923</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>2923</v>
+        <v>2924</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="3" t="s">
-        <v>2919</v>
+        <v>2920</v>
       </c>
       <c r="B5" s="3">
         <v>4</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>2924</v>
+        <v>2925</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>2925</v>
+        <v>2926</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B6" s="3">
         <v>5</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>2927</v>
+        <v>2928</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>2928</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B7" s="3">
         <v>6</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>2929</v>
+        <v>2930</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>2930</v>
+        <v>2931</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B8" s="3">
         <v>7</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>2931</v>
+        <v>2932</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>2932</v>
+        <v>2933</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B9" s="3">
         <v>8</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>2933</v>
+        <v>2934</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>2934</v>
+        <v>2935</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B10" s="3">
         <v>9</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>2935</v>
+        <v>2936</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>2936</v>
+        <v>2937</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B11" s="3">
         <v>10</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>2937</v>
+        <v>2938</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>2938</v>
+        <v>2939</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B12" s="3">
         <v>11</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>2939</v>
+        <v>2940</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>2940</v>
+        <v>2941</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B13" s="3">
         <v>12</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>2941</v>
+        <v>2942</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>2942</v>
+        <v>2943</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B14" s="3">
         <v>13</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>2943</v>
+        <v>2944</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>2944</v>
+        <v>2945</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="3" t="s">
-        <v>2926</v>
+        <v>2927</v>
       </c>
       <c r="B15" s="3">
         <v>14</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>2945</v>
+        <v>2946</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>2946</v>
+        <v>2947</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="3" t="s">
-        <v>2947</v>
+        <v>2948</v>
       </c>
       <c r="B16" s="3">
         <v>16</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>2948</v>
+        <v>2949</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>2949</v>
+        <v>2950</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="3" t="s">
-        <v>2947</v>
+        <v>2948</v>
       </c>
       <c r="B17" s="3">
         <v>17</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>2950</v>
+        <v>2951</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>2951</v>
+        <v>2952</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="3" t="s">
-        <v>2947</v>
+        <v>2948</v>
       </c>
       <c r="B18" s="3">
         <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>2952</v>
+        <v>2953</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>2953</v>
+        <v>2954</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="3" t="s">
-        <v>2954</v>
+        <v>2955</v>
       </c>
       <c r="B19" s="3">
         <v>19</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>2955</v>
+        <v>2956</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>2956</v>
+        <v>2957</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="3" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="B20" s="3">
         <v>20</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>2958</v>
+        <v>2959</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>2959</v>
+        <v>2960</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="3" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="B21" s="3">
         <v>21</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>2960</v>
+        <v>2961</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>2961</v>
+        <v>2962</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="3" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="B22" s="3">
         <v>22</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>2962</v>
+        <v>2963</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>2963</v>
+        <v>2964</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="3" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="B23" s="3">
         <v>23</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>2964</v>
+        <v>2965</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>2965</v>
+        <v>2966</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="3" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="B24" s="3">
         <v>26</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>2966</v>
+        <v>2967</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>2967</v>
+        <v>2968</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="3" t="s">
+        <v>2969</v>
+      </c>
+      <c r="B25" s="3">
+        <v>27</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>2970</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>2971</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D24"/>
+  <autoFilter ref="A1:D25"/>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Date" prompt="YYYY-MM-DD" sqref="A2:A2001"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Plan version" prompt="From 1, one per change." sqref="B2:B2001"/>

</xml_diff>